<commit_message>
AMZN rescore 2026-10-05: R3 4->3, M2 4->3 (Dom-approved); +SBGSY enters
Objective inputs refreshed (price-driven). Subjective review against the
Q2 2026 10-Q:
- R3: long-term debt $68.8B -> $133.0B in six months, TTM FCF negative,
  $137B leases not yet commenced; consistent with the META precedent.
- M2: 126-day return in line with SPY (+18.1% vs +18.2%).
- Rule-15 EPS-YoY blank for the 2026-06-30 quarter recorded in
  eps-yoy-overrides.json (ruling dated 2026-08-02).
Score 73.9 -> 73.6; tradable rank 15 -> 16 (hold band). SBGSY enters at
rank 15: model event 'membership: +SBGSY', 17 holdings at equal weight.
Rating Audit rows 3032-3034. Thesis allocation headers updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-09-18 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-10-05 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-09-18, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-10-05, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J5" t="inlineStr"/>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -1287,16 +1287,16 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>79.15000000000001</v>
+        <v>79.25</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1318,23 +1318,23 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>79</v>
+        <v>79.15000000000001</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
@@ -1512,23 +1512,23 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RDDT</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>75.39</v>
+        <v>75.23</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1550,9 +1550,13 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>6.25</v>
-      </c>
-      <c r="J13" t="inlineStr"/>
+        <v>5.88</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1566,7 +1570,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>75.26000000000001</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1588,78 +1592,74 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>6861.T</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>75.23</v>
+        <v>74.62</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>13</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="n">
-        <v>6.25</v>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>6861.T</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>74.62</v>
+        <v>74.43000000000001</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="E16" t="n">
+        <v>13</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
+      <c r="I16" t="n">
+        <v>5.88</v>
+      </c>
       <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1674,7 +1674,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>74.58</v>
+        <v>74.42</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1696,23 +1696,23 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>73.88</v>
+        <v>73.65000000000001</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>ENTER (rank 15, score 73.6)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1734,14 +1734,14 @@
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1750,7 +1750,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>73.08</v>
+        <v>73.62</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J19" t="inlineStr"/>
     </row>
@@ -1810,16 +1810,16 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>RDDT</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>72.47</v>
+        <v>72.64</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1829,28 +1829,35 @@
       <c r="E21" t="n">
         <v>18</v>
       </c>
-      <c r="F21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
+      <c r="I21" t="n">
+        <v>5.88</v>
+      </c>
       <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>71.93000000000001</v>
+        <v>72.47</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1872,16 +1879,16 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>70.98</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1891,11 +1898,7 @@
       <c r="E23" t="n">
         <v>20</v>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>EXIT (pending since 2026-09-08, confirmed)</t>
-        </is>
-      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>N</t>
@@ -1907,16 +1910,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>70.78</v>
+        <v>71.38</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1938,16 +1941,16 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>NTAP</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>70.7</v>
+        <v>70.98</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1969,16 +1972,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>70.23999999999999</v>
+        <v>70.78</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2000,20 +2003,20 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>69.88</v>
+        <v>70.7</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -2040,11 +2043,11 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>69.56</v>
+        <v>70.53</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -2062,20 +2065,20 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CGNX</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>69.53</v>
+        <v>70.23999999999999</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -2093,16 +2096,16 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>CGNX</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>69.5</v>
+        <v>69.53</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2124,16 +2127,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>69.31999999999999</v>
+        <v>69.5</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2155,21 +2158,24 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>6268.T</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>69.18000000000001</v>
+        <v>69.31999999999999</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E32" t="n">
+        <v>29</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
@@ -2183,24 +2189,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>6268.T</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>69.11</v>
+        <v>69.18000000000001</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E33" t="n">
-        <v>29</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
@@ -2209,30 +2212,29 @@
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
-        </is>
-      </c>
+      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BSL.DE</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>68.56999999999999</v>
+        <v>69.11</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E34" t="n">
+        <v>30</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
@@ -2241,21 +2243,25 @@
         </is>
       </c>
       <c r="H34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>68.48999999999999</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2263,7 +2269,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
@@ -2277,24 +2283,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>BSL.DE</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>68.43000000000001</v>
+        <v>68.56999999999999</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E36" t="n">
-        <v>31</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
@@ -2308,16 +2311,16 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>68.42</v>
+        <v>68.48999999999999</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2339,16 +2342,16 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>68.20999999999999</v>
+        <v>68.43000000000001</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2370,16 +2373,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>68.2</v>
+        <v>68.42</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2396,25 +2399,21 @@
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
-        </is>
-      </c>
+      <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>HSAI</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>67.89</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2436,16 +2435,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>67.84999999999999</v>
+        <v>68.2</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2462,21 +2461,25 @@
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>HSAI</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>67.43000000000001</v>
+        <v>67.89</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2498,16 +2501,16 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>67.13</v>
+        <v>67.84999999999999</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2529,16 +2532,16 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>67.13</v>
+        <v>67.43000000000001</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2560,16 +2563,16 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>67.05</v>
+        <v>67.13</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2591,16 +2594,16 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>66.81</v>
+        <v>67.13</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2622,16 +2625,16 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>66.8</v>
+        <v>66.81</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2653,16 +2656,16 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>RRC</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>66.79000000000001</v>
+        <v>66.8</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2684,16 +2687,16 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>RRC</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>66.75</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2715,16 +2718,16 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>66.7</v>
+        <v>66.75</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2991,16 +2994,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>65.79000000000001</v>
+        <v>65.81999999999999</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3017,25 +3020,21 @@
         </is>
       </c>
       <c r="H59" t="inlineStr"/>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
-        </is>
-      </c>
+      <c r="J59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>PLAB</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>65.7</v>
+        <v>65.79000000000001</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3052,12 +3051,16 @@
         </is>
       </c>
       <c r="H60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>PLAB</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3066,7 +3069,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>65.68000000000001</v>
+        <v>65.7</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -3088,16 +3091,16 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>65.63</v>
+        <v>65.68000000000001</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3150,7 +3153,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3159,7 +3162,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>65.56</v>
+        <v>65.52</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3212,16 +3215,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>65.22</v>
+        <v>65.25</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3238,25 +3241,21 @@
         </is>
       </c>
       <c r="H66" t="inlineStr"/>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
+      <c r="J66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>65.12</v>
+        <v>65.22</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3273,7 +3272,11 @@
         </is>
       </c>
       <c r="H67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3287,7 +3290,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>65.01000000000001</v>
+        <v>65.16</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3399,16 +3402,16 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>64.81</v>
+        <v>64.88</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3430,7 +3433,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3439,7 +3442,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>64.79000000000001</v>
+        <v>64.81999999999999</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3461,16 +3464,16 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>MKSI</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>64.72</v>
+        <v>64.81</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -3492,7 +3495,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>MKSI</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3501,7 +3504,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>64.08</v>
+        <v>64.72</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3523,16 +3526,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>63.74</v>
+        <v>64.08</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3554,16 +3557,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>63.6</v>
+        <v>63.74</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3585,16 +3588,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>63.58</v>
+        <v>63.6</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3616,16 +3619,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>GNRC</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>63.53</v>
+        <v>63.58</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3647,16 +3650,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>63.5</v>
+        <v>63.53</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3678,16 +3681,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>UMAC</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>63.48</v>
+        <v>63.5</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3709,16 +3712,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SYM</t>
+          <t>UMAC</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>63.28</v>
+        <v>63.48</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3740,16 +3743,16 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>HIVE</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>63.26</v>
+        <v>63.38</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3771,16 +3774,16 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>SYM</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>63.21</v>
+        <v>63.28</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -3802,21 +3805,24 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2252.HK</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>63.15</v>
+        <v>63.26</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E85" t="n">
+        <v>78</v>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
@@ -3830,16 +3836,16 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>HIVE</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>63.12</v>
+        <v>63.21</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3847,7 +3853,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
@@ -3861,24 +3867,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>2252.HK</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>63.12</v>
+        <v>63.15</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E87" t="n">
-        <v>79</v>
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
@@ -3892,16 +3895,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>63.09</v>
+        <v>63.12</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3923,16 +3926,16 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>62.97</v>
+        <v>63.09</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3954,16 +3957,16 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>62.79</v>
+        <v>62.89</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -4078,16 +4081,16 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>62.54</v>
+        <v>62.39</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -4109,16 +4112,16 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>62.39</v>
+        <v>62.38</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -4140,16 +4143,16 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>06 AI Compute Silicon / Programmable logic</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>62.38</v>
+        <v>62.28</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -4171,16 +4174,16 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Programmable logic</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>62.28</v>
+        <v>62.26</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -4202,16 +4205,16 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>62.26</v>
+        <v>62.25</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -4233,24 +4236,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>6383.T</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>62.25</v>
+        <v>61.91</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E99" t="n">
-        <v>91</v>
       </c>
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
@@ -4264,21 +4264,24 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>6383.T</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>61.91</v>
+        <v>61.79</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E100" t="n">
+        <v>91</v>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
@@ -4292,16 +4295,16 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>61.79</v>
+        <v>61.65</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4323,16 +4326,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>SPCX</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>61.65</v>
+        <v>61.57</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4354,16 +4357,16 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SPCX</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>61.57</v>
+        <v>61.42</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -4385,24 +4388,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>2590.HK</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>61.53</v>
+        <v>61.41</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E104" t="n">
-        <v>95</v>
       </c>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
@@ -4416,16 +4416,16 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>61.45</v>
+        <v>61.36</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -4433,7 +4433,7 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
@@ -4442,21 +4442,25 @@
         </is>
       </c>
       <c r="H105" t="inlineStr"/>
-      <c r="J105" t="inlineStr"/>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>61.42</v>
+        <v>61.31</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4464,7 +4468,7 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
@@ -4478,21 +4482,24 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2590.HK</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>10 Models, Software &amp; Applications / Financial software</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>61.41</v>
+        <v>61.29</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E107" t="n">
+        <v>97</v>
       </c>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
@@ -4506,16 +4513,16 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>NOVT</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>61.36</v>
+        <v>61.17</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -4532,25 +4539,21 @@
         </is>
       </c>
       <c r="H108" t="inlineStr"/>
-      <c r="J108" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
-        </is>
-      </c>
+      <c r="J108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Financial software</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>61.29</v>
+        <v>61.14</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -4572,16 +4575,16 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>NOVT</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>61.17</v>
+        <v>61.04</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -4603,16 +4606,16 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>AMKR</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>61.14</v>
+        <v>60.95</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -4634,16 +4637,16 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>61.04</v>
+        <v>60.91</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -4665,16 +4668,16 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>AMKR</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>60.95</v>
+        <v>60.91</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -4696,16 +4699,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>60.91</v>
+        <v>60.85</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4736,7 +4739,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>60.86</v>
+        <v>60.74</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -4758,16 +4761,16 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>PRCT</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>60.85</v>
+        <v>60.61</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -4789,16 +4792,16 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>PRCT</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>60.61</v>
+        <v>60.54</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -4820,16 +4823,16 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>60.54</v>
+        <v>60.47</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -4851,16 +4854,16 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>60.47</v>
+        <v>60.42</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -4882,16 +4885,16 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>60.45</v>
+        <v>60.38</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -4913,16 +4916,16 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>10 Models, Software &amp; Applications / Consumer fintech (AI adopter)</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>60.42</v>
+        <v>60.33</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -4944,16 +4947,16 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>60.38</v>
+        <v>60.3</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -4975,16 +4978,16 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Consumer fintech (AI adopter)</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>60.33</v>
+        <v>60.25</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -5006,16 +5009,16 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>60.3</v>
+        <v>60.01</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -5037,16 +5040,16 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>MBLY</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>60.25</v>
+        <v>59.94</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -5068,16 +5071,16 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>MBLY</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>59.94</v>
+        <v>59.65</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -5108,7 +5111,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>59.77</v>
+        <v>59.6</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -5127,16 +5130,16 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>WDAY</t>
+          <t>TKR</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>59.65</v>
+        <v>59.49</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -5158,12 +5161,12 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>TKR</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -5220,16 +5223,16 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>AVAV</t>
+          <t>TOELY</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>59.42</v>
+        <v>59.26</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -5251,16 +5254,16 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>TOELY</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>59.26</v>
+        <v>59.12</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
@@ -5282,16 +5285,16 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>RRX</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>58.88</v>
+        <v>58.84</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
@@ -5313,16 +5316,16 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>RRX</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>58.84</v>
+        <v>58.73</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
@@ -5344,16 +5347,16 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>58.73</v>
+        <v>58.7</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -5375,16 +5378,16 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>ASX</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>58.7</v>
+        <v>58.67</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
@@ -5406,16 +5409,16 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>ASX</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>58.67</v>
+        <v>58.53</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
@@ -5437,24 +5440,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>6506.T</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>58.53</v>
+        <v>58.52</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E138" t="n">
-        <v>127</v>
       </c>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
@@ -5468,21 +5468,24 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>6506.T</t>
+          <t>ONDS</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>58.52</v>
+        <v>58.32</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E139" t="n">
+        <v>127</v>
       </c>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
@@ -5496,16 +5499,16 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>ONDS</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>58.48</v>
+        <v>58.22</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
@@ -5527,16 +5530,16 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>58.22</v>
+        <v>58.02</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -5558,16 +5561,16 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>58.02</v>
+        <v>57.97</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
@@ -5589,16 +5592,16 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>10 Models, Software &amp; Applications / AI data layer</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>57.97</v>
+        <v>57.76</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -5620,24 +5623,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>2049.TW</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI data layer</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>57.76</v>
+        <v>57.75</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E144" t="n">
-        <v>132</v>
       </c>
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
@@ -5651,21 +5651,24 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2049.TW</t>
+          <t>TNC</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>11 Robotics &amp; Physical AI / Humanoid &amp; service robot makers</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>57.75</v>
+        <v>57.67</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E145" t="n">
+        <v>132</v>
       </c>
       <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
@@ -5679,24 +5682,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>TNC</t>
+          <t>DRO.AX</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Humanoid &amp; service robot makers</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>57.67</v>
+        <v>57.64</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E146" t="n">
-        <v>133</v>
       </c>
       <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
@@ -5710,21 +5710,24 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>DRO.AX</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>57.64</v>
+        <v>57.57</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E147" t="n">
+        <v>133</v>
       </c>
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
@@ -5738,16 +5741,16 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>57.57</v>
+        <v>57.38</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
@@ -5769,16 +5772,16 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>CAMT</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>57.38</v>
+        <v>57.12</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
@@ -5800,16 +5803,16 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>CAMT</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>57.12</v>
+        <v>56.98</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
@@ -5831,16 +5834,16 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PSIX</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>56.98</v>
+        <v>56.61</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
@@ -5862,16 +5865,16 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>PSIX</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>56.61</v>
+        <v>56.44</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -5893,16 +5896,16 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>TEM</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>56.44</v>
+        <v>56.12</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -5924,24 +5927,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>TEM</t>
+          <t>6481.T</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>56.12</v>
+        <v>56.01</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E154" t="n">
-        <v>140</v>
       </c>
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
@@ -5955,21 +5955,24 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>6481.T</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>56.01</v>
+        <v>55.94</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E155" t="n">
+        <v>140</v>
       </c>
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
@@ -5983,16 +5986,16 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>ATKR</t>
+          <t>AVAV</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>55.97</v>
+        <v>55.73</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
@@ -6014,16 +6017,16 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>ATKR</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>55.94</v>
+        <v>55.49</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(rule 30): block OTC ADRs the broker can't fill; SBGSY exits the model
The tradability filter only rejected exchange-suffix tickers, so SBGSY (an
OTC ADR) entered at rank 15 on 2026-10-05 and the broker returned 'not
found'. is_tradable now also rejects portfolio_sizing.BROKER_UNTRADABLE:
not listed (SBGSY, ABBNY, TOELY, HHUSF) and whole-share only (HTHIY, BESIY).
Model event 'membership: -SBGSY'; back to 16 holdings at 6.25%. Scores,
ratings and Watchlist membership unchanged. CLAUDE.md rule 30 amended
(Dom-approved). No seam stamped: a constraint cannot start an exit clock.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J5" t="inlineStr"/>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J7" t="inlineStr"/>
     </row>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
@@ -1658,7 +1658,7 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J17" t="inlineStr"/>
     </row>
@@ -1712,30 +1712,24 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>73.65000000000001</v>
+        <v>73.76000000000001</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>15</v>
-      </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>ENTER (rank 15, score 73.6)</t>
+          <t>EXIT (untradable)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="n">
-        <v>5.88</v>
-      </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1758,7 +1752,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1772,7 +1766,7 @@
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J19" t="inlineStr"/>
     </row>
@@ -1796,7 +1790,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
@@ -1827,7 +1821,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1841,7 +1835,7 @@
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J21" t="inlineStr"/>
     </row>
@@ -1865,7 +1859,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
@@ -1896,7 +1890,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
@@ -1927,7 +1921,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
@@ -1958,7 +1952,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
@@ -1989,7 +1983,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
@@ -2020,7 +2014,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
@@ -2050,9 +2044,6 @@
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E28" t="n">
-        <v>25</v>
-      </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
@@ -2082,7 +2073,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
@@ -2113,7 +2104,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
@@ -2144,7 +2135,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
@@ -2175,7 +2166,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
@@ -2234,7 +2225,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
@@ -2269,7 +2260,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
@@ -2328,7 +2319,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
@@ -2359,7 +2350,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
@@ -2390,7 +2381,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
@@ -2421,7 +2412,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
@@ -2452,7 +2443,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
@@ -2487,7 +2478,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
@@ -2518,7 +2509,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
@@ -2549,7 +2540,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
@@ -2580,7 +2571,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
@@ -2611,7 +2602,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
@@ -2642,7 +2633,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
@@ -2673,7 +2664,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
@@ -2704,7 +2695,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
@@ -2735,7 +2726,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
@@ -2766,7 +2757,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
@@ -2825,7 +2816,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
@@ -2856,7 +2847,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
@@ -2887,7 +2878,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
@@ -2918,7 +2909,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
@@ -2949,7 +2940,7 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
@@ -2980,7 +2971,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
@@ -3011,7 +3002,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
@@ -3042,7 +3033,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
@@ -3077,7 +3068,7 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
@@ -3108,7 +3099,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
@@ -3139,7 +3130,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
@@ -3170,7 +3161,7 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
@@ -3201,7 +3192,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
@@ -3232,7 +3223,7 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
@@ -3263,7 +3254,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
@@ -3298,7 +3289,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
@@ -3357,7 +3348,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
@@ -3388,7 +3379,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
@@ -3419,7 +3410,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
@@ -3449,9 +3440,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E73" t="n">
-        <v>66</v>
-      </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
@@ -3481,7 +3469,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
@@ -3512,7 +3500,7 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
@@ -3543,7 +3531,7 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
@@ -3574,7 +3562,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
@@ -3604,9 +3592,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E78" t="n">
-        <v>71</v>
-      </c>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
@@ -3636,7 +3621,7 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
@@ -3667,7 +3652,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
@@ -3698,7 +3683,7 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
@@ -3729,7 +3714,7 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
@@ -3760,7 +3745,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
@@ -3791,7 +3776,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
@@ -3822,7 +3807,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
@@ -3853,7 +3838,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
@@ -3912,7 +3897,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
@@ -3943,7 +3928,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
@@ -3974,7 +3959,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
@@ -4005,7 +3990,7 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
@@ -4036,7 +4021,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
@@ -4067,7 +4052,7 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
@@ -4098,7 +4083,7 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
@@ -4129,7 +4114,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
@@ -4160,7 +4145,7 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
@@ -4191,7 +4176,7 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
@@ -4222,7 +4207,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
@@ -4281,7 +4266,7 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
@@ -4312,7 +4297,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
@@ -4343,7 +4328,7 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
@@ -4374,7 +4359,7 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
@@ -4433,7 +4418,7 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
@@ -4468,7 +4453,7 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
@@ -4499,7 +4484,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
@@ -4530,7 +4515,7 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
@@ -4561,7 +4546,7 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
@@ -4592,7 +4577,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
@@ -4623,7 +4608,7 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
@@ -4654,7 +4639,7 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
@@ -4685,7 +4670,7 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
@@ -4716,7 +4701,7 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
@@ -4747,7 +4732,7 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
@@ -4778,7 +4763,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
@@ -4809,7 +4794,7 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
@@ -4840,7 +4825,7 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
@@ -4871,7 +4856,7 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
@@ -4902,7 +4887,7 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
@@ -4933,7 +4918,7 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
@@ -4964,7 +4949,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
@@ -4995,7 +4980,7 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
@@ -5026,7 +5011,7 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
@@ -5057,7 +5042,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
@@ -5088,7 +5073,7 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
@@ -5147,7 +5132,7 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
@@ -5161,16 +5146,16 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>ALNT</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>59.49</v>
+        <v>59.45</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
@@ -5178,7 +5163,7 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
@@ -5192,24 +5177,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ALNT</t>
+          <t>TOELY</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>59.45</v>
+        <v>59.26</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E130" t="n">
-        <v>119</v>
       </c>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
@@ -5223,16 +5205,16 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>TOELY</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>59.26</v>
+        <v>59.12</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -5240,7 +5222,7 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
@@ -5254,12 +5236,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -5271,7 +5253,7 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
@@ -5302,7 +5284,7 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
@@ -5333,7 +5315,7 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
@@ -5364,7 +5346,7 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
@@ -5395,7 +5377,7 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
@@ -5426,7 +5408,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
@@ -5485,7 +5467,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
@@ -5516,7 +5498,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
@@ -5547,7 +5529,7 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
@@ -5578,7 +5560,7 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
@@ -5609,7 +5591,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
@@ -5668,7 +5650,7 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
@@ -5727,7 +5709,7 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
@@ -5758,7 +5740,7 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr">
@@ -5789,7 +5771,7 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr">
@@ -5820,7 +5802,7 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
@@ -5851,7 +5833,7 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
@@ -5882,7 +5864,7 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
@@ -5913,7 +5895,7 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
@@ -5972,7 +5954,7 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
@@ -6003,7 +5985,7 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
@@ -6034,7 +6016,7 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
@@ -6065,7 +6047,7 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">

</xml_diff>

<commit_message>
fix(rule 30): block OTC ADRs the broker can't fill; SBGSY exits the model (#98)
The tradability filter only rejected exchange-suffix tickers, so SBGSY (an
OTC ADR) entered at rank 15 on 2026-10-05 and the broker returned 'not
found'. is_tradable now also rejects portfolio_sizing.BROKER_UNTRADABLE:
not listed (SBGSY, ABBNY, TOELY, HHUSF) and whole-share only (HTHIY, BESIY).
Model event 'membership: -SBGSY'; back to 16 holdings at 6.25%. Scores,
ratings and Watchlist membership unchanged. CLAUDE.md rule 30 amended
(Dom-approved). No seam stamped: a constraint cannot start an exit clock.

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J5" t="inlineStr"/>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J7" t="inlineStr"/>
     </row>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
@@ -1658,7 +1658,7 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J17" t="inlineStr"/>
     </row>
@@ -1712,30 +1712,24 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>73.65000000000001</v>
+        <v>73.76000000000001</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>15</v>
-      </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>ENTER (rank 15, score 73.6)</t>
+          <t>EXIT (untradable)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="n">
-        <v>5.88</v>
-      </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1758,7 +1752,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1772,7 +1766,7 @@
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J19" t="inlineStr"/>
     </row>
@@ -1796,7 +1790,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
@@ -1827,7 +1821,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1841,7 +1835,7 @@
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J21" t="inlineStr"/>
     </row>
@@ -1865,7 +1859,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
@@ -1896,7 +1890,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
@@ -1927,7 +1921,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
@@ -1958,7 +1952,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
@@ -1989,7 +1983,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
@@ -2020,7 +2014,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
@@ -2050,9 +2044,6 @@
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E28" t="n">
-        <v>25</v>
-      </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
@@ -2082,7 +2073,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
@@ -2113,7 +2104,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
@@ -2144,7 +2135,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
@@ -2175,7 +2166,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
@@ -2234,7 +2225,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
@@ -2269,7 +2260,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
@@ -2328,7 +2319,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
@@ -2359,7 +2350,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
@@ -2390,7 +2381,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
@@ -2421,7 +2412,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
@@ -2452,7 +2443,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
@@ -2487,7 +2478,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
@@ -2518,7 +2509,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
@@ -2549,7 +2540,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
@@ -2580,7 +2571,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
@@ -2611,7 +2602,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
@@ -2642,7 +2633,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
@@ -2673,7 +2664,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
@@ -2704,7 +2695,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
@@ -2735,7 +2726,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
@@ -2766,7 +2757,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
@@ -2825,7 +2816,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
@@ -2856,7 +2847,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
@@ -2887,7 +2878,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
@@ -2918,7 +2909,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
@@ -2949,7 +2940,7 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
@@ -2980,7 +2971,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
@@ -3011,7 +3002,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
@@ -3042,7 +3033,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
@@ -3077,7 +3068,7 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
@@ -3108,7 +3099,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
@@ -3139,7 +3130,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
@@ -3170,7 +3161,7 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
@@ -3201,7 +3192,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
@@ -3232,7 +3223,7 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
@@ -3263,7 +3254,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
@@ -3298,7 +3289,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
@@ -3357,7 +3348,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
@@ -3388,7 +3379,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
@@ -3419,7 +3410,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
@@ -3449,9 +3440,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E73" t="n">
-        <v>66</v>
-      </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
@@ -3481,7 +3469,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
@@ -3512,7 +3500,7 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
@@ -3543,7 +3531,7 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
@@ -3574,7 +3562,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
@@ -3604,9 +3592,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E78" t="n">
-        <v>71</v>
-      </c>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
@@ -3636,7 +3621,7 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
@@ -3667,7 +3652,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
@@ -3698,7 +3683,7 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
@@ -3729,7 +3714,7 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
@@ -3760,7 +3745,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
@@ -3791,7 +3776,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
@@ -3822,7 +3807,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
@@ -3853,7 +3838,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
@@ -3912,7 +3897,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
@@ -3943,7 +3928,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
@@ -3974,7 +3959,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
@@ -4005,7 +3990,7 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
@@ -4036,7 +4021,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
@@ -4067,7 +4052,7 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
@@ -4098,7 +4083,7 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
@@ -4129,7 +4114,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
@@ -4160,7 +4145,7 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
@@ -4191,7 +4176,7 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
@@ -4222,7 +4207,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
@@ -4281,7 +4266,7 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
@@ -4312,7 +4297,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
@@ -4343,7 +4328,7 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
@@ -4374,7 +4359,7 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
@@ -4433,7 +4418,7 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
@@ -4468,7 +4453,7 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
@@ -4499,7 +4484,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
@@ -4530,7 +4515,7 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
@@ -4561,7 +4546,7 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
@@ -4592,7 +4577,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
@@ -4623,7 +4608,7 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
@@ -4654,7 +4639,7 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
@@ -4685,7 +4670,7 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
@@ -4716,7 +4701,7 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
@@ -4747,7 +4732,7 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
@@ -4778,7 +4763,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
@@ -4809,7 +4794,7 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
@@ -4840,7 +4825,7 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
@@ -4871,7 +4856,7 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
@@ -4902,7 +4887,7 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
@@ -4933,7 +4918,7 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
@@ -4964,7 +4949,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
@@ -4995,7 +4980,7 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
@@ -5026,7 +5011,7 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
@@ -5057,7 +5042,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
@@ -5088,7 +5073,7 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
@@ -5147,7 +5132,7 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
@@ -5161,16 +5146,16 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>ALNT</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>59.49</v>
+        <v>59.45</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
@@ -5178,7 +5163,7 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
@@ -5192,24 +5177,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ALNT</t>
+          <t>TOELY</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>59.45</v>
+        <v>59.26</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E130" t="n">
-        <v>119</v>
       </c>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
@@ -5223,16 +5205,16 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>TOELY</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>59.26</v>
+        <v>59.12</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -5240,7 +5222,7 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
@@ -5254,12 +5236,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -5271,7 +5253,7 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
@@ -5302,7 +5284,7 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
@@ -5333,7 +5315,7 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
@@ -5364,7 +5346,7 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
@@ -5395,7 +5377,7 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
@@ -5426,7 +5408,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
@@ -5485,7 +5467,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
@@ -5516,7 +5498,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
@@ -5547,7 +5529,7 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
@@ -5578,7 +5560,7 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
@@ -5609,7 +5591,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
@@ -5668,7 +5650,7 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
@@ -5727,7 +5709,7 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
@@ -5758,7 +5740,7 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr">
@@ -5789,7 +5771,7 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr">
@@ -5820,7 +5802,7 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
@@ -5851,7 +5833,7 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
@@ -5882,7 +5864,7 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
@@ -5913,7 +5895,7 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
@@ -5972,7 +5954,7 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
@@ -6003,7 +5985,7 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
@@ -6034,7 +6016,7 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
@@ -6065,7 +6047,7 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">

</xml_diff>

<commit_message>
rating-research 2026-10-18: ANET/FIX/SNDK/MSFT briefed, 9 proposals; AMZN exit (ticket held)
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-11 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-10-18 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J162"/>
+  <dimension ref="A1:J164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1068,7 +1068,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-10-11, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-10-18, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
@@ -1174,7 +1174,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>82.25</v>
+        <v>82.38</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J4" t="inlineStr"/>
     </row>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -1245,16 +1245,16 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>81.44</v>
+        <v>81.58</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1276,27 +1276,27 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>81.25</v>
+        <v>81.44</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1318,11 +1318,11 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
+          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
@@ -1452,7 +1452,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>78.27</v>
+        <v>78.77</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1474,23 +1474,23 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>75.3</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1512,51 +1512,61 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>6861.T</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>74.28</v>
+        <v>75.8</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
+      <c r="E13" t="n">
+        <v>11</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
+      <c r="I13" t="n">
+        <v>5.88</v>
+      </c>
       <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GMED</t>
+          <t>RDDT</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>73.92</v>
+        <v>75.53</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1564,7 +1574,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1578,93 +1588,89 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>6861.T</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>73.67</v>
+        <v>74.28</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>12</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="n">
-        <v>5.56</v>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>GMED</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>73.51000000000001</v>
+        <v>73.92</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="E16" t="n">
+        <v>13</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
+      <c r="I16" t="n">
+        <v>5.88</v>
+      </c>
       <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>73.48</v>
+        <v>73.91</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1672,7 +1678,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1686,23 +1692,23 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>73.31</v>
+        <v>73.75</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1710,75 +1716,62 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>ENTER (rank 14, score 73.3)</t>
+          <t>ENTRY DEFERRED (rank 15, score 73.8; entry hold until 2026-11-15: San Diego County enforcement action filed 2026-10-05 (People v. AppLovin, seeks an injunction on data collection) and securities class action Talbot v. AppLovin, 3:26-cv-10584 (N.D. Cal., filed 2026-09-16); growth decelerating with Q3 uplift untested)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="n">
-        <v>5.56</v>
-      </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>73</v>
+        <v>73.51000000000001</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>15</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>ENTER (rank 15, score 73.0)</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="n">
-        <v>5.56</v>
-      </c>
       <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>03 DC Infrastructure</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>72.75</v>
+        <v>73.48</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1800,23 +1793,23 @@
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RDDT</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>03 DC Infrastructure</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>72.7</v>
+        <v>73.25</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1838,23 +1831,23 @@
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>72.65000000000001</v>
+        <v>73.17</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1864,14 +1857,25 @@
       <c r="E22" t="n">
         <v>18</v>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
+      <c r="I22" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1885,7 +1889,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>72.48999999999999</v>
+        <v>72.98999999999999</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1907,16 +1911,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>72.25</v>
+        <v>72.65000000000001</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1926,35 +1930,28 @@
       <c r="E24" t="n">
         <v>20</v>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>EXIT PENDING (rank 20 &gt; exit rank 18, since 2026-10-11)</t>
-        </is>
-      </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="I24" t="n">
-        <v>5.56</v>
-      </c>
       <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>72.23999999999999</v>
+        <v>72.38</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1976,16 +1973,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>71.93000000000001</v>
+        <v>72.25</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1995,7 +1992,11 @@
       <c r="E26" t="n">
         <v>22</v>
       </c>
-      <c r="F26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>EXIT (pending since 2026-10-11, confirmed)</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
           <t>N</t>
@@ -2007,16 +2008,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>71.88</v>
+        <v>72.23999999999999</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2069,16 +2070,16 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>71.58</v>
+        <v>71.81999999999999</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2100,21 +2101,24 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BSL.DE</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>70.95999999999999</v>
+        <v>71.81</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
+      </c>
+      <c r="E30" t="n">
+        <v>26</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
@@ -2128,16 +2132,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>70.45</v>
+        <v>71.58</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2145,7 +2149,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
@@ -2159,24 +2163,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>BSL.DE</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>70.23</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
-      </c>
-      <c r="E32" t="n">
-        <v>27</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
@@ -2190,16 +2191,16 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>70</v>
+        <v>70.23</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2221,20 +2222,20 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>69.95999999999999</v>
+        <v>70.19</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -2252,16 +2253,16 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>69.65000000000001</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2283,16 +2284,16 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CGNX</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>69.26000000000001</v>
+        <v>69.53</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2314,24 +2315,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>HTHIY</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>69.23999999999999</v>
+        <v>69.17</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E37" t="n">
-        <v>32</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
@@ -2345,21 +2343,24 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>HTHIY</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>69.17</v>
+        <v>69.15000000000001</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E38" t="n">
+        <v>32</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
@@ -2373,16 +2374,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>69.15000000000001</v>
+        <v>68.89</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2404,16 +2405,16 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>CGNX</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>69</v>
+        <v>68.88</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2435,16 +2436,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>68.73</v>
+        <v>68.86</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2466,16 +2467,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>NTAP</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>68.67</v>
+        <v>68.73</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2497,16 +2498,16 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>68.45999999999999</v>
+        <v>68.67</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2528,16 +2529,16 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>68.31999999999999</v>
+        <v>68.45999999999999</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2554,25 +2555,21 @@
         </is>
       </c>
       <c r="H44" t="inlineStr"/>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
-        </is>
-      </c>
+      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>NOVT</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>68.12</v>
+        <v>68.31999999999999</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2589,21 +2586,25 @@
         </is>
       </c>
       <c r="H45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>NOVT</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>68.11</v>
+        <v>68.12</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2625,16 +2626,16 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>68.02</v>
+        <v>68.11</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2656,21 +2657,24 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>6268.T</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>67.98</v>
+        <v>68</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E48" t="n">
+        <v>42</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
@@ -2684,24 +2688,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>6268.T</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>67.87</v>
+        <v>67.98</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E49" t="n">
-        <v>42</v>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
@@ -2715,7 +2716,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2724,7 +2725,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>67.59999999999999</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2746,16 +2747,16 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>67.42</v>
+        <v>67.7</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2772,30 +2773,29 @@
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
-        </is>
-      </c>
+      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>6954.T</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>67.33</v>
+        <v>67.42</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E52" t="n">
+        <v>45</v>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
@@ -2804,29 +2804,30 @@
         </is>
       </c>
       <c r="H52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>6954.T</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>67.31</v>
+        <v>67.33</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E53" t="n">
-        <v>45</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
@@ -2840,16 +2841,16 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>67.22</v>
+        <v>67.31</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2871,16 +2872,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>67.15000000000001</v>
+        <v>67.22</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2902,16 +2903,16 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>67.13</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -2964,16 +2965,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
+          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>66.51000000000001</v>
+        <v>67</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2995,21 +2996,24 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>AUTO.OL</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>66.51000000000001</v>
+        <v>66.89</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E59" t="n">
+        <v>51</v>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
@@ -3023,16 +3027,16 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>65.97</v>
+        <v>66.72</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3040,7 +3044,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
@@ -3054,24 +3058,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>AUTO.OL</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>65.73</v>
+        <v>66.51000000000001</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E61" t="n">
-        <v>52</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
@@ -3085,16 +3086,16 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>65.73</v>
+        <v>66.02</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3116,16 +3117,16 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>65.61</v>
+        <v>65.97</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3147,16 +3148,16 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>65.43000000000001</v>
+        <v>65.95999999999999</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3178,16 +3179,16 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>65.40000000000001</v>
+        <v>65.73</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3209,16 +3210,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>65.38</v>
+        <v>65.73</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3240,16 +3241,16 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>65.29000000000001</v>
+        <v>65.48999999999999</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3271,16 +3272,16 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>65.25</v>
+        <v>65.38</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3302,16 +3303,16 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>OUST</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>65.20999999999999</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3333,21 +3334,24 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>65.19</v>
+        <v>65.25</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E70" t="n">
+        <v>61</v>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
@@ -3361,16 +3365,16 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>OUST</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>65.04000000000001</v>
+        <v>65.20999999999999</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3378,7 +3382,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
@@ -3392,16 +3396,16 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>64.94</v>
+        <v>65.04000000000001</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3409,7 +3413,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
@@ -3423,16 +3427,16 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>64.94</v>
+        <v>65.02</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3440,7 +3444,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
@@ -3449,25 +3453,21 @@
         </is>
       </c>
       <c r="H73" t="inlineStr"/>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
+      <c r="J73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>64.75</v>
+        <v>65.02</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -3475,7 +3475,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
@@ -3489,24 +3489,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>64.73</v>
+        <v>64.87</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E75" t="n">
-        <v>65</v>
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
@@ -3520,16 +3517,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>64.52</v>
+        <v>64.75</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3551,16 +3548,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>64.43000000000001</v>
+        <v>64.73</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3582,16 +3579,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>64.34</v>
+        <v>64.56999999999999</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3613,16 +3610,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>64.31</v>
+        <v>64.52</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3644,16 +3641,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Programmable logic</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>64.29000000000001</v>
+        <v>64.47</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3670,21 +3667,25 @@
         </is>
       </c>
       <c r="H80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>GNRC</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>64.28</v>
+        <v>64.44</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3706,16 +3707,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>64.13</v>
+        <v>64.43000000000001</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3737,7 +3738,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>PLAB</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3746,7 +3747,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>64.08</v>
+        <v>64.31</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3768,16 +3769,16 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>UMAC</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>63.86</v>
+        <v>64.28</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -3799,16 +3800,16 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>63.84</v>
+        <v>64.15000000000001</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -3825,26 +3826,33 @@
         </is>
       </c>
       <c r="H85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>TOELY</t>
+          <t>PLAB</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>63.84</v>
+        <v>64.08</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E86" t="n">
+        <v>76</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
@@ -3858,21 +3866,24 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>63.78</v>
+        <v>64.06</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E87" t="n">
+        <v>77</v>
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
@@ -3886,16 +3897,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>06 AI Compute Silicon / Programmable logic</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>63.58</v>
+        <v>63.92</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3903,7 +3914,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
@@ -3917,16 +3928,16 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>UMAC</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>63.04</v>
+        <v>63.86</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3934,7 +3945,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
@@ -3948,16 +3959,16 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>63</v>
+        <v>63.84</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -3965,7 +3976,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
@@ -3974,33 +3985,26 @@
         </is>
       </c>
       <c r="H90" t="inlineStr"/>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
-        </is>
-      </c>
+      <c r="J90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>TOELY</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>62.77</v>
+        <v>63.84</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E91" t="n">
-        <v>79</v>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
@@ -4014,24 +4018,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>SYM</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>62.74</v>
+        <v>63.78</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E92" t="n">
-        <v>80</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
@@ -4045,21 +4046,24 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>6383.T</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>62.59</v>
+        <v>63.63</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E93" t="n">
+        <v>81</v>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
@@ -4073,16 +4077,16 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>62.47</v>
+        <v>63.28</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -4090,7 +4094,7 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
@@ -4104,16 +4108,16 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>62.45</v>
+        <v>63</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -4121,7 +4125,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
@@ -4132,23 +4136,23 @@
       <c r="H95" t="inlineStr"/>
       <c r="J95" t="inlineStr">
         <is>
-          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
+          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>10 Models, Software &amp; Applications / Financial software</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>62.35</v>
+        <v>62.83</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -4156,7 +4160,7 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
@@ -4170,16 +4174,16 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>SYM</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Financial software</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>62.33</v>
+        <v>62.74</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -4187,7 +4191,7 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
@@ -4201,24 +4205,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>6383.T</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>62.25</v>
+        <v>62.59</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E98" t="n">
-        <v>85</v>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
@@ -4232,21 +4233,24 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2252.HK</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>62.1</v>
+        <v>62.47</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E99" t="n">
+        <v>86</v>
       </c>
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
@@ -4260,16 +4264,16 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>KTOS</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>62.06</v>
+        <v>62.35</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -4277,7 +4281,7 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
@@ -4291,16 +4295,16 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>62.02</v>
+        <v>62.27</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4308,7 +4312,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
@@ -4322,16 +4326,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>HSAI</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>61.98</v>
+        <v>62.25</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4339,7 +4343,7 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
@@ -4353,24 +4357,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>2252.HK</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>61.58</v>
+        <v>62.1</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E103" t="n">
-        <v>89</v>
       </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
@@ -4384,16 +4385,16 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>KTOS</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>61.57</v>
+        <v>62.06</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -4415,16 +4416,16 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>HSAI</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>61.47</v>
+        <v>61.98</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -4446,16 +4447,16 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>61.46</v>
+        <v>61.58</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4477,16 +4478,16 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>61.3</v>
+        <v>61.47</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4508,16 +4509,16 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>MBLY</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>61.3</v>
+        <v>61.42</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -4539,16 +4540,16 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>61.05</v>
+        <v>61.3</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -4570,16 +4571,16 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>60.89</v>
+        <v>61.05</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -4601,21 +4602,24 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2049.TW</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>60.8</v>
+        <v>60.89</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E111" t="n">
+        <v>97</v>
       </c>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
@@ -4629,16 +4633,16 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>WDAY</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>60.67</v>
+        <v>60.86</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -4646,7 +4650,7 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
@@ -4660,7 +4664,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>RRX</t>
+          <t>2049.TW</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -4669,15 +4673,12 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>60.61</v>
+        <v>60.8</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E113" t="n">
-        <v>98</v>
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
@@ -4691,16 +4692,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>MBLY</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>60.6</v>
+        <v>60.7</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4722,16 +4723,16 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>RRX</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>60.51</v>
+        <v>60.61</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -4753,16 +4754,16 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>60.46</v>
+        <v>60.6</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -4784,16 +4785,16 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>RRC</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>60.18</v>
+        <v>60.58</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -4815,16 +4816,16 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>60.07</v>
+        <v>60.46</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -4846,16 +4847,16 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>SPCX</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>60.04</v>
+        <v>60.27</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -4877,16 +4878,16 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>59.83</v>
+        <v>60.2</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -4908,16 +4909,16 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>PRCT</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>59.77</v>
+        <v>60.07</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -4939,16 +4940,16 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>SPCX</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>59.7</v>
+        <v>59.85</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -4970,16 +4971,16 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>AMKR</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>59.57</v>
+        <v>59.83</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -5001,16 +5002,16 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>PRCT</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>59.29</v>
+        <v>59.77</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -5032,21 +5033,24 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>6506.T</t>
+          <t>RRC</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>59.23</v>
+        <v>59.69</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E125" t="n">
+        <v>110</v>
       </c>
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
@@ -5060,16 +5064,16 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>AMKR</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>59</v>
+        <v>59.57</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -5077,7 +5081,7 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
@@ -5091,24 +5095,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ALNT</t>
+          <t>6506.T</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>58.88</v>
+        <v>59.23</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E127" t="n">
-        <v>111</v>
       </c>
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
@@ -5122,21 +5123,24 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>6481.T</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>10 Models, Software &amp; Applications / AI data layer</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>58.88</v>
+        <v>59.21</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E128" t="n">
+        <v>112</v>
       </c>
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
@@ -5150,16 +5154,16 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>58.77</v>
+        <v>59</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
@@ -5167,7 +5171,7 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
@@ -5181,16 +5185,16 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>ALNT</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Consumer fintech (AI adopter)</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>58.75</v>
+        <v>58.88</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -5198,7 +5202,7 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
@@ -5212,16 +5216,16 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>KGX.DE</t>
+          <t>6481.T</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>58.72</v>
+        <v>58.88</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -5240,16 +5244,16 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI data layer</t>
+          <t>10 Models, Software &amp; Applications / AI commerce</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>58.59</v>
+        <v>58.84</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
@@ -5257,7 +5261,7 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
@@ -5271,24 +5275,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>KGX.DE</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>58.48</v>
+        <v>58.72</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E133" t="n">
-        <v>115</v>
       </c>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
@@ -5302,16 +5303,16 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>UPST</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>58.41</v>
+        <v>58.68</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
@@ -5333,16 +5334,16 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>58.33</v>
+        <v>58.48</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -5364,16 +5365,16 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>58.18</v>
+        <v>58.4</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
@@ -5395,16 +5396,16 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>ASX</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>58.04</v>
+        <v>58.33</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
@@ -5426,16 +5427,16 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>58.01</v>
+        <v>58.18</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
@@ -5457,16 +5458,16 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>ONDS</t>
+          <t>ASX</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>57.95</v>
+        <v>58.04</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
@@ -5488,16 +5489,16 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>57.89</v>
+        <v>58.01</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
@@ -5519,16 +5520,16 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>WYFI</t>
+          <t>ONDS</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>57.67</v>
+        <v>57.95</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -5550,21 +5551,24 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>DRO.AX</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>57.49</v>
+        <v>57.89</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E142" t="n">
+        <v>124</v>
       </c>
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
@@ -5578,16 +5582,16 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>WYFI</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>57.44</v>
+        <v>57.67</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -5595,7 +5599,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
@@ -5609,24 +5613,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>CARR</t>
+          <t>DRO.AX</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>57.44</v>
+        <v>57.49</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E144" t="n">
-        <v>125</v>
       </c>
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
@@ -5640,16 +5641,16 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>CARR</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>57.11</v>
+        <v>57.44</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
@@ -5671,16 +5672,16 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>HIVE</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>57</v>
+        <v>57.32</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
@@ -5702,16 +5703,16 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>TKR</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>10 Models, Software &amp; Applications / Consumer fintech (AI adopter)</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>56.86</v>
+        <v>57.15</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
@@ -5733,16 +5734,16 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>AVAV</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>56.81</v>
+        <v>57.12</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
@@ -5764,16 +5765,16 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>56.71</v>
+        <v>57.11</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
@@ -5795,16 +5796,16 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>TKR</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>56.66</v>
+        <v>56.86</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
@@ -5826,16 +5827,16 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>TNC</t>
+          <t>AVAV</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Humanoid &amp; service robot makers</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>56.59</v>
+        <v>56.81</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
@@ -5857,16 +5858,16 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>56.21</v>
+        <v>56.71</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -5888,16 +5889,16 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>PPL</t>
+          <t>HIVE</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>56.14</v>
+        <v>56.62</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -5919,16 +5920,16 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>55.95</v>
+        <v>56.21</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -5950,16 +5951,16 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>PSIX</t>
+          <t>TNC</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>11 Robotics &amp; Physical AI / Humanoid &amp; service robot makers</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>55.93</v>
+        <v>56.21</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
@@ -5981,16 +5982,16 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>UCTT</t>
+          <t>PPL</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>55.86</v>
+        <v>56.02</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
@@ -6012,21 +6013,24 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>6324.T</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>55.69</v>
+        <v>55.95</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E157" t="n">
+        <v>138</v>
       </c>
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
@@ -6040,7 +6044,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>BW</t>
+          <t>PSIX</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -6049,7 +6053,7 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>55.67</v>
+        <v>55.93</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
@@ -6057,7 +6061,7 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
@@ -6071,16 +6075,16 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>UCTT</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>55.29</v>
+        <v>55.86</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
@@ -6088,7 +6092,7 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
@@ -6102,16 +6106,16 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2590.HK</t>
+          <t>6324.T</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>55.27</v>
+        <v>55.69</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
@@ -6130,16 +6134,16 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>APLD</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>55.25</v>
+        <v>55.29</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
@@ -6147,7 +6151,7 @@
         </is>
       </c>
       <c r="E161" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
@@ -6161,24 +6165,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>2590.HK</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>55.14</v>
+        <v>55.27</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E162" t="n">
-        <v>141</v>
       </c>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
@@ -6188,6 +6189,68 @@
       </c>
       <c r="H162" t="inlineStr"/>
       <c r="J162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>01 Power Generation / Distributed / on-site power</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>55.17</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>142</v>
+      </c>
+      <c r="F163" t="inlineStr"/>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr"/>
+      <c r="J163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>AEP</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>55.14</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>143</v>
+      </c>
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr"/>
+      <c r="J164" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
rating-research 2026-10-18: ANET/FIX/SNDK/MSFT briefed, 9 proposals; AMZN exit (ticket held) (#170)
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-11 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-10-18 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J162"/>
+  <dimension ref="A1:J164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1068,7 +1068,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-10-11, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-10-18, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
@@ -1174,7 +1174,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>82.25</v>
+        <v>82.38</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J4" t="inlineStr"/>
     </row>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -1245,16 +1245,16 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>81.44</v>
+        <v>81.58</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1276,27 +1276,27 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>81.25</v>
+        <v>81.44</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1318,11 +1318,11 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
+          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
@@ -1452,7 +1452,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>78.27</v>
+        <v>78.77</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1474,23 +1474,23 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>75.3</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1512,51 +1512,61 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>6861.T</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>74.28</v>
+        <v>75.8</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
+      <c r="E13" t="n">
+        <v>11</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
+      <c r="I13" t="n">
+        <v>5.88</v>
+      </c>
       <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GMED</t>
+          <t>RDDT</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>73.92</v>
+        <v>75.53</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1564,7 +1574,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1578,93 +1588,89 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>6861.T</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>73.67</v>
+        <v>74.28</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>12</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="n">
-        <v>5.56</v>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>GMED</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>73.51000000000001</v>
+        <v>73.92</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="E16" t="n">
+        <v>13</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
+      <c r="I16" t="n">
+        <v>5.88</v>
+      </c>
       <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>73.48</v>
+        <v>73.91</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1672,7 +1678,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1686,23 +1692,23 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>73.31</v>
+        <v>73.75</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1710,75 +1716,62 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>ENTER (rank 14, score 73.3)</t>
+          <t>ENTRY DEFERRED (rank 15, score 73.8; entry hold until 2026-11-15: San Diego County enforcement action filed 2026-10-05 (People v. AppLovin, seeks an injunction on data collection) and securities class action Talbot v. AppLovin, 3:26-cv-10584 (N.D. Cal., filed 2026-09-16); growth decelerating with Q3 uplift untested)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="n">
-        <v>5.56</v>
-      </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>73</v>
+        <v>73.51000000000001</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>15</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>ENTER (rank 15, score 73.0)</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="n">
-        <v>5.56</v>
-      </c>
       <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>03 DC Infrastructure</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>72.75</v>
+        <v>73.48</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1800,23 +1793,23 @@
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RDDT</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>03 DC Infrastructure</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>72.7</v>
+        <v>73.25</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1838,23 +1831,23 @@
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>72.65000000000001</v>
+        <v>73.17</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1864,14 +1857,25 @@
       <c r="E22" t="n">
         <v>18</v>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
+      <c r="I22" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1885,7 +1889,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>72.48999999999999</v>
+        <v>72.98999999999999</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1907,16 +1911,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>72.25</v>
+        <v>72.65000000000001</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1926,35 +1930,28 @@
       <c r="E24" t="n">
         <v>20</v>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>EXIT PENDING (rank 20 &gt; exit rank 18, since 2026-10-11)</t>
-        </is>
-      </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="I24" t="n">
-        <v>5.56</v>
-      </c>
       <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>72.23999999999999</v>
+        <v>72.38</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1976,16 +1973,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>71.93000000000001</v>
+        <v>72.25</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1995,7 +1992,11 @@
       <c r="E26" t="n">
         <v>22</v>
       </c>
-      <c r="F26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>EXIT (pending since 2026-10-11, confirmed)</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
           <t>N</t>
@@ -2007,16 +2008,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>71.88</v>
+        <v>72.23999999999999</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2069,16 +2070,16 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>71.58</v>
+        <v>71.81999999999999</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2100,21 +2101,24 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BSL.DE</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>70.95999999999999</v>
+        <v>71.81</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
+      </c>
+      <c r="E30" t="n">
+        <v>26</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
@@ -2128,16 +2132,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>70.45</v>
+        <v>71.58</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2145,7 +2149,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
@@ -2159,24 +2163,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>BSL.DE</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>70.23</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
-      </c>
-      <c r="E32" t="n">
-        <v>27</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
@@ -2190,16 +2191,16 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>70</v>
+        <v>70.23</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2221,20 +2222,20 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>69.95999999999999</v>
+        <v>70.19</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -2252,16 +2253,16 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>69.65000000000001</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2283,16 +2284,16 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CGNX</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>69.26000000000001</v>
+        <v>69.53</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2314,24 +2315,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>HTHIY</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>69.23999999999999</v>
+        <v>69.17</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E37" t="n">
-        <v>32</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
@@ -2345,21 +2343,24 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>HTHIY</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>69.17</v>
+        <v>69.15000000000001</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E38" t="n">
+        <v>32</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
@@ -2373,16 +2374,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>69.15000000000001</v>
+        <v>68.89</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2404,16 +2405,16 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>CGNX</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>69</v>
+        <v>68.88</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2435,16 +2436,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>68.73</v>
+        <v>68.86</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2466,16 +2467,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>NTAP</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>68.67</v>
+        <v>68.73</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2497,16 +2498,16 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>68.45999999999999</v>
+        <v>68.67</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2528,16 +2529,16 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>68.31999999999999</v>
+        <v>68.45999999999999</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2554,25 +2555,21 @@
         </is>
       </c>
       <c r="H44" t="inlineStr"/>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
-        </is>
-      </c>
+      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>NOVT</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>68.12</v>
+        <v>68.31999999999999</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2589,21 +2586,25 @@
         </is>
       </c>
       <c r="H45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>NOVT</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>68.11</v>
+        <v>68.12</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2625,16 +2626,16 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>68.02</v>
+        <v>68.11</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2656,21 +2657,24 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>6268.T</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>67.98</v>
+        <v>68</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E48" t="n">
+        <v>42</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
@@ -2684,24 +2688,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>6268.T</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>67.87</v>
+        <v>67.98</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E49" t="n">
-        <v>42</v>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
@@ -2715,7 +2716,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2724,7 +2725,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>67.59999999999999</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2746,16 +2747,16 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>67.42</v>
+        <v>67.7</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2772,30 +2773,29 @@
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
-        </is>
-      </c>
+      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>6954.T</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>67.33</v>
+        <v>67.42</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E52" t="n">
+        <v>45</v>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
@@ -2804,29 +2804,30 @@
         </is>
       </c>
       <c r="H52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>6954.T</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>67.31</v>
+        <v>67.33</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E53" t="n">
-        <v>45</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
@@ -2840,16 +2841,16 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>67.22</v>
+        <v>67.31</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2871,16 +2872,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>67.15000000000001</v>
+        <v>67.22</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2902,16 +2903,16 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>67.13</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -2964,16 +2965,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
+          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>66.51000000000001</v>
+        <v>67</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2995,21 +2996,24 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>AUTO.OL</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>66.51000000000001</v>
+        <v>66.89</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E59" t="n">
+        <v>51</v>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
@@ -3023,16 +3027,16 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>65.97</v>
+        <v>66.72</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3040,7 +3044,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
@@ -3054,24 +3058,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>AUTO.OL</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>65.73</v>
+        <v>66.51000000000001</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E61" t="n">
-        <v>52</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
@@ -3085,16 +3086,16 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>65.73</v>
+        <v>66.02</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3116,16 +3117,16 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>65.61</v>
+        <v>65.97</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3147,16 +3148,16 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>65.43000000000001</v>
+        <v>65.95999999999999</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3178,16 +3179,16 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>65.40000000000001</v>
+        <v>65.73</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3209,16 +3210,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>65.38</v>
+        <v>65.73</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3240,16 +3241,16 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>65.29000000000001</v>
+        <v>65.48999999999999</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3271,16 +3272,16 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>65.25</v>
+        <v>65.38</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3302,16 +3303,16 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>OUST</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>65.20999999999999</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3333,21 +3334,24 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>65.19</v>
+        <v>65.25</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E70" t="n">
+        <v>61</v>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
@@ -3361,16 +3365,16 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>OUST</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>65.04000000000001</v>
+        <v>65.20999999999999</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3378,7 +3382,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
@@ -3392,16 +3396,16 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>64.94</v>
+        <v>65.04000000000001</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3409,7 +3413,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
@@ -3423,16 +3427,16 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>64.94</v>
+        <v>65.02</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3440,7 +3444,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
@@ -3449,25 +3453,21 @@
         </is>
       </c>
       <c r="H73" t="inlineStr"/>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
+      <c r="J73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>64.75</v>
+        <v>65.02</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -3475,7 +3475,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
@@ -3489,24 +3489,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>64.73</v>
+        <v>64.87</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E75" t="n">
-        <v>65</v>
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
@@ -3520,16 +3517,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>64.52</v>
+        <v>64.75</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3551,16 +3548,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>64.43000000000001</v>
+        <v>64.73</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3582,16 +3579,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>64.34</v>
+        <v>64.56999999999999</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3613,16 +3610,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>64.31</v>
+        <v>64.52</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3644,16 +3641,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Programmable logic</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>64.29000000000001</v>
+        <v>64.47</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3670,21 +3667,25 @@
         </is>
       </c>
       <c r="H80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>GNRC</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>64.28</v>
+        <v>64.44</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3706,16 +3707,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>64.13</v>
+        <v>64.43000000000001</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3737,7 +3738,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>PLAB</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3746,7 +3747,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>64.08</v>
+        <v>64.31</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3768,16 +3769,16 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>UMAC</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>63.86</v>
+        <v>64.28</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -3799,16 +3800,16 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>63.84</v>
+        <v>64.15000000000001</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -3825,26 +3826,33 @@
         </is>
       </c>
       <c r="H85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>TOELY</t>
+          <t>PLAB</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>63.84</v>
+        <v>64.08</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E86" t="n">
+        <v>76</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
@@ -3858,21 +3866,24 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>63.78</v>
+        <v>64.06</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E87" t="n">
+        <v>77</v>
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
@@ -3886,16 +3897,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>06 AI Compute Silicon / Programmable logic</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>63.58</v>
+        <v>63.92</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3903,7 +3914,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
@@ -3917,16 +3928,16 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>UMAC</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>63.04</v>
+        <v>63.86</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3934,7 +3945,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
@@ -3948,16 +3959,16 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>63</v>
+        <v>63.84</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -3965,7 +3976,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
@@ -3974,33 +3985,26 @@
         </is>
       </c>
       <c r="H90" t="inlineStr"/>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
-        </is>
-      </c>
+      <c r="J90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>TOELY</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>62.77</v>
+        <v>63.84</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E91" t="n">
-        <v>79</v>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
@@ -4014,24 +4018,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>SYM</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>62.74</v>
+        <v>63.78</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E92" t="n">
-        <v>80</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
@@ -4045,21 +4046,24 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>6383.T</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>62.59</v>
+        <v>63.63</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E93" t="n">
+        <v>81</v>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
@@ -4073,16 +4077,16 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>62.47</v>
+        <v>63.28</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -4090,7 +4094,7 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
@@ -4104,16 +4108,16 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>62.45</v>
+        <v>63</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -4121,7 +4125,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
@@ -4132,23 +4136,23 @@
       <c r="H95" t="inlineStr"/>
       <c r="J95" t="inlineStr">
         <is>
-          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
+          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>10 Models, Software &amp; Applications / Financial software</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>62.35</v>
+        <v>62.83</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -4156,7 +4160,7 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
@@ -4170,16 +4174,16 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>SYM</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Financial software</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>62.33</v>
+        <v>62.74</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -4187,7 +4191,7 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
@@ -4201,24 +4205,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>6383.T</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>62.25</v>
+        <v>62.59</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E98" t="n">
-        <v>85</v>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
@@ -4232,21 +4233,24 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2252.HK</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>62.1</v>
+        <v>62.47</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E99" t="n">
+        <v>86</v>
       </c>
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
@@ -4260,16 +4264,16 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>KTOS</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>62.06</v>
+        <v>62.35</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -4277,7 +4281,7 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
@@ -4291,16 +4295,16 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>62.02</v>
+        <v>62.27</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4308,7 +4312,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
@@ -4322,16 +4326,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>HSAI</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>61.98</v>
+        <v>62.25</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4339,7 +4343,7 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
@@ -4353,24 +4357,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>2252.HK</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>61.58</v>
+        <v>62.1</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E103" t="n">
-        <v>89</v>
       </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
@@ -4384,16 +4385,16 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>KTOS</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>61.57</v>
+        <v>62.06</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -4415,16 +4416,16 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>HSAI</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>61.47</v>
+        <v>61.98</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -4446,16 +4447,16 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>61.46</v>
+        <v>61.58</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4477,16 +4478,16 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>61.3</v>
+        <v>61.47</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4508,16 +4509,16 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>MBLY</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>61.3</v>
+        <v>61.42</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -4539,16 +4540,16 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>61.05</v>
+        <v>61.3</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -4570,16 +4571,16 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>60.89</v>
+        <v>61.05</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -4601,21 +4602,24 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2049.TW</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>60.8</v>
+        <v>60.89</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E111" t="n">
+        <v>97</v>
       </c>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
@@ -4629,16 +4633,16 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>WDAY</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>60.67</v>
+        <v>60.86</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -4646,7 +4650,7 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
@@ -4660,7 +4664,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>RRX</t>
+          <t>2049.TW</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -4669,15 +4673,12 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>60.61</v>
+        <v>60.8</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E113" t="n">
-        <v>98</v>
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
@@ -4691,16 +4692,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>MBLY</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>60.6</v>
+        <v>60.7</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4722,16 +4723,16 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>RRX</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>60.51</v>
+        <v>60.61</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -4753,16 +4754,16 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>60.46</v>
+        <v>60.6</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -4784,16 +4785,16 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>RRC</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>60.18</v>
+        <v>60.58</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -4815,16 +4816,16 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>60.07</v>
+        <v>60.46</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -4846,16 +4847,16 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>SPCX</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>60.04</v>
+        <v>60.27</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -4877,16 +4878,16 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>59.83</v>
+        <v>60.2</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -4908,16 +4909,16 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>PRCT</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>59.77</v>
+        <v>60.07</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -4939,16 +4940,16 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>SPCX</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>59.7</v>
+        <v>59.85</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -4970,16 +4971,16 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>AMKR</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>59.57</v>
+        <v>59.83</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -5001,16 +5002,16 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>PRCT</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>59.29</v>
+        <v>59.77</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -5032,21 +5033,24 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>6506.T</t>
+          <t>RRC</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>59.23</v>
+        <v>59.69</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E125" t="n">
+        <v>110</v>
       </c>
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
@@ -5060,16 +5064,16 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>AMKR</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>59</v>
+        <v>59.57</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -5077,7 +5081,7 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
@@ -5091,24 +5095,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ALNT</t>
+          <t>6506.T</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>58.88</v>
+        <v>59.23</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E127" t="n">
-        <v>111</v>
       </c>
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
@@ -5122,21 +5123,24 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>6481.T</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>10 Models, Software &amp; Applications / AI data layer</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>58.88</v>
+        <v>59.21</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E128" t="n">
+        <v>112</v>
       </c>
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
@@ -5150,16 +5154,16 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>58.77</v>
+        <v>59</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
@@ -5167,7 +5171,7 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
@@ -5181,16 +5185,16 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>ALNT</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Consumer fintech (AI adopter)</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>58.75</v>
+        <v>58.88</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -5198,7 +5202,7 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
@@ -5212,16 +5216,16 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>KGX.DE</t>
+          <t>6481.T</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>58.72</v>
+        <v>58.88</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -5240,16 +5244,16 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI data layer</t>
+          <t>10 Models, Software &amp; Applications / AI commerce</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>58.59</v>
+        <v>58.84</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
@@ -5257,7 +5261,7 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
@@ -5271,24 +5275,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>KGX.DE</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>58.48</v>
+        <v>58.72</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E133" t="n">
-        <v>115</v>
       </c>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
@@ -5302,16 +5303,16 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>UPST</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>58.41</v>
+        <v>58.68</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
@@ -5333,16 +5334,16 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>58.33</v>
+        <v>58.48</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -5364,16 +5365,16 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>58.18</v>
+        <v>58.4</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
@@ -5395,16 +5396,16 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>ASX</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>58.04</v>
+        <v>58.33</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
@@ -5426,16 +5427,16 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>58.01</v>
+        <v>58.18</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
@@ -5457,16 +5458,16 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>ONDS</t>
+          <t>ASX</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>57.95</v>
+        <v>58.04</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
@@ -5488,16 +5489,16 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>57.89</v>
+        <v>58.01</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
@@ -5519,16 +5520,16 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>WYFI</t>
+          <t>ONDS</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>57.67</v>
+        <v>57.95</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -5550,21 +5551,24 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>DRO.AX</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>57.49</v>
+        <v>57.89</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E142" t="n">
+        <v>124</v>
       </c>
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
@@ -5578,16 +5582,16 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>WYFI</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>57.44</v>
+        <v>57.67</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -5595,7 +5599,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
@@ -5609,24 +5613,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>CARR</t>
+          <t>DRO.AX</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>57.44</v>
+        <v>57.49</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E144" t="n">
-        <v>125</v>
       </c>
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
@@ -5640,16 +5641,16 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>CARR</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>57.11</v>
+        <v>57.44</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
@@ -5671,16 +5672,16 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>HIVE</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>57</v>
+        <v>57.32</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
@@ -5702,16 +5703,16 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>TKR</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>10 Models, Software &amp; Applications / Consumer fintech (AI adopter)</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>56.86</v>
+        <v>57.15</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
@@ -5733,16 +5734,16 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>AVAV</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>56.81</v>
+        <v>57.12</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
@@ -5764,16 +5765,16 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>56.71</v>
+        <v>57.11</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
@@ -5795,16 +5796,16 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>TKR</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>56.66</v>
+        <v>56.86</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
@@ -5826,16 +5827,16 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>TNC</t>
+          <t>AVAV</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Humanoid &amp; service robot makers</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>56.59</v>
+        <v>56.81</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
@@ -5857,16 +5858,16 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>56.21</v>
+        <v>56.71</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -5888,16 +5889,16 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>PPL</t>
+          <t>HIVE</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>56.14</v>
+        <v>56.62</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -5919,16 +5920,16 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>55.95</v>
+        <v>56.21</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -5950,16 +5951,16 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>PSIX</t>
+          <t>TNC</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>11 Robotics &amp; Physical AI / Humanoid &amp; service robot makers</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>55.93</v>
+        <v>56.21</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
@@ -5981,16 +5982,16 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>UCTT</t>
+          <t>PPL</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>55.86</v>
+        <v>56.02</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
@@ -6012,21 +6013,24 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>6324.T</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>55.69</v>
+        <v>55.95</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E157" t="n">
+        <v>138</v>
       </c>
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
@@ -6040,7 +6044,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>BW</t>
+          <t>PSIX</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -6049,7 +6053,7 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>55.67</v>
+        <v>55.93</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
@@ -6057,7 +6061,7 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
@@ -6071,16 +6075,16 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>UCTT</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>55.29</v>
+        <v>55.86</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
@@ -6088,7 +6092,7 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
@@ -6102,16 +6106,16 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2590.HK</t>
+          <t>6324.T</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>55.27</v>
+        <v>55.69</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
@@ -6130,16 +6134,16 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>APLD</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>55.25</v>
+        <v>55.29</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
@@ -6147,7 +6151,7 @@
         </is>
       </c>
       <c r="E161" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
@@ -6161,24 +6165,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>2590.HK</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>55.14</v>
+        <v>55.27</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E162" t="n">
-        <v>141</v>
       </c>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
@@ -6188,6 +6189,68 @@
       </c>
       <c r="H162" t="inlineStr"/>
       <c r="J162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>01 Power Generation / Distributed / on-site power</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>55.17</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>142</v>
+      </c>
+      <c r="F163" t="inlineStr"/>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr"/>
+      <c r="J163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>AEP</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>55.14</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>143</v>
+      </c>
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr"/>
+      <c r="J164" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
daily-watch 2026-10-26: FIX/WDC/LRCX re-scored; EME+VRT exit, LRCX enters; ticket HELD
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-18 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-10-26 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J164"/>
+  <dimension ref="A1:J163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1068,7 +1068,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-10-18, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-10-26, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1127,20 +1127,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>84.39</v>
+        <v>85.83</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓✓✓</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1158,23 +1158,27 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J3" t="inlineStr"/>
+        <v>6.25</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>82.38</v>
+        <v>83.87</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1196,23 +1200,23 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>81.90000000000001</v>
+        <v>82.38</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1234,27 +1238,23 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
-        </is>
-      </c>
+        <v>6.25</v>
+      </c>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>81.58</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1276,27 +1276,27 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
+          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>81.44</v>
+        <v>81.58</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1318,18 +1318,18 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1360,23 +1360,23 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>79.53</v>
+        <v>79.79000000000001</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1398,23 +1398,23 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>79.40000000000001</v>
+        <v>79.53</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1436,23 +1436,23 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06 Silicon - Memory</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>78.77</v>
+        <v>79.15000000000001</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1474,23 +1474,23 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>06 Silicon - Memory</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>76.40000000000001</v>
+        <v>78.39</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1512,23 +1512,23 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>75.8</v>
+        <v>76.27</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1550,23 +1550,23 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RDDT</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>75.53</v>
+        <v>75.8</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1588,51 +1588,61 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>6861.T</t>
+          <t>RDDT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>74.28</v>
+        <v>75.53</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
+      <c r="E15" t="n">
+        <v>13</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>6.25</v>
+      </c>
       <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GMED</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>73.92</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1640,7 +1650,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1654,61 +1664,51 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>6861.T</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>73.91</v>
+        <v>74.28</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E17" t="n">
-        <v>14</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="n">
-        <v>5.88</v>
-      </c>
       <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>73.75</v>
+        <v>74.03</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1720,58 +1720,71 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>ENTRY DEFERRED (rank 15, score 73.8; entry hold until 2026-11-15: San Diego County enforcement action filed 2026-10-05 (People v. AppLovin, seeks an injunction on data collection) and securities class action Talbot v. AppLovin, 3:26-cv-10584 (N.D. Cal., filed 2026-09-16); growth decelerating with Q3 uplift untested)</t>
+          <t>ENTER (rank 15, score 74.0)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
+      <c r="I18" t="n">
+        <v>6.25</v>
+      </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>GMED</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>73.51000000000001</v>
+        <v>73.92</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>16</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
+      <c r="I19" t="n">
+        <v>6.25</v>
+      </c>
       <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>73.48</v>
+        <v>73.75</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1779,75 +1792,58 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>16</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="n">
-        <v>5.88</v>
-      </c>
       <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>03 DC Infrastructure</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>73.25</v>
+        <v>73.51000000000001</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E21" t="n">
-        <v>17</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="n">
-        <v>5.88</v>
-      </c>
       <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>73.17</v>
+        <v>73.27</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1857,25 +1853,14 @@
       <c r="E22" t="n">
         <v>18</v>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1911,16 +1896,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>72.65000000000001</v>
+        <v>72.87</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1937,21 +1922,25 @@
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>03 DC Infrastructure</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>72.38</v>
+        <v>72.75</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1973,16 +1962,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>72.25</v>
+        <v>72.38</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1992,11 +1981,7 @@
       <c r="E26" t="n">
         <v>22</v>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>EXIT (pending since 2026-10-11, confirmed)</t>
-        </is>
-      </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>N</t>
@@ -2008,16 +1993,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>72.23999999999999</v>
+        <v>72.25</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2070,16 +2055,16 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>71.81999999999999</v>
+        <v>71.86</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2101,16 +2086,16 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>71.81</v>
+        <v>71.58</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2132,16 +2117,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>71.58</v>
+        <v>71.45</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2163,21 +2148,24 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BSL.DE</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>70.95999999999999</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
+      </c>
+      <c r="E32" t="n">
+        <v>28</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
@@ -2191,24 +2179,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>BSL.DE</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>70.23</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
-      </c>
-      <c r="E33" t="n">
-        <v>28</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
@@ -2222,16 +2207,16 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>70.19</v>
+        <v>70.68000000000001</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2253,16 +2238,16 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>69.95999999999999</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2284,24 +2269,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>HTHIY</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>69.53</v>
+        <v>69.17</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E36" t="n">
-        <v>31</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
@@ -2315,12 +2297,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>HTHIY</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -2331,6 +2313,9 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="E37" t="n">
+        <v>31</v>
+      </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
@@ -2374,16 +2359,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>CGNX</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>68.89</v>
+        <v>68.88</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2405,16 +2390,16 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CGNX</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>68.88</v>
+        <v>68.86</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2436,16 +2421,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>68.86</v>
+        <v>68.45999999999999</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2467,16 +2452,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>68.73</v>
+        <v>68.45999999999999</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2498,16 +2483,16 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>68.67</v>
+        <v>68.31999999999999</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2524,21 +2509,25 @@
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>NTAP</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>68.45999999999999</v>
+        <v>68.31</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2560,16 +2549,16 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>NOVT</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>68.31999999999999</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2586,25 +2575,21 @@
         </is>
       </c>
       <c r="H45" t="inlineStr"/>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
-        </is>
-      </c>
+      <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>NOVT</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>68.12</v>
+        <v>68</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2626,24 +2611,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>6268.T</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>68.11</v>
+        <v>67.98</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E47" t="n">
-        <v>41</v>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
@@ -2657,16 +2639,16 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>68</v>
+        <v>67.95</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2674,7 +2656,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
@@ -2688,21 +2670,24 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>6268.T</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>67.98</v>
+        <v>67.73</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E49" t="n">
+        <v>42</v>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
@@ -2716,16 +2701,16 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>67.90000000000001</v>
+        <v>67.7</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2747,16 +2732,16 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>67.7</v>
+        <v>67.42</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2773,21 +2758,25 @@
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>67.42</v>
+        <v>67.22</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -2804,30 +2793,29 @@
         </is>
       </c>
       <c r="H52" t="inlineStr"/>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
-        </is>
-      </c>
+      <c r="J52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>6954.T</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>67.33</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E53" t="n">
+        <v>46</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
@@ -2841,16 +2829,16 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>MKSI</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>67.31</v>
+        <v>67</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2858,7 +2846,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
@@ -2872,16 +2860,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>67.22</v>
+        <v>67</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2889,7 +2877,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
@@ -2903,7 +2891,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2912,7 +2900,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>67.15000000000001</v>
+        <v>66.93000000000001</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -2920,7 +2908,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
@@ -2934,24 +2922,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MKSI</t>
+          <t>6954.T</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>67.12</v>
+        <v>66.83</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E57" t="n">
-        <v>49</v>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
@@ -2965,16 +2950,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>WDAY</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>67</v>
+        <v>66.73</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2996,16 +2981,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>66.89</v>
+        <v>66.72</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3027,16 +3012,16 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>66.72</v>
+        <v>66.27</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3058,21 +3043,24 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>AUTO.OL</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>66.51000000000001</v>
+        <v>66.20999999999999</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E61" t="n">
+        <v>53</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
@@ -3086,24 +3074,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>AUTO.OL</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>66.02</v>
+        <v>66.13</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E62" t="n">
-        <v>53</v>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
@@ -3117,16 +3102,16 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>65.97</v>
+        <v>66.02</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3179,16 +3164,16 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>65.73</v>
+        <v>65.67</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3210,16 +3195,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>65.73</v>
+        <v>65.61</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3241,16 +3226,16 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>65.48999999999999</v>
+        <v>65.31</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3272,16 +3257,16 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>OUST</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>65.38</v>
+        <v>65.20999999999999</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3303,16 +3288,16 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>65.29000000000001</v>
+        <v>65.04000000000001</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3334,16 +3319,16 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>65.25</v>
+        <v>65.02</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3365,16 +3350,16 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>OUST</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>65.20999999999999</v>
+        <v>64.88</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3396,16 +3381,16 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>65.04000000000001</v>
+        <v>64.75</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3427,16 +3412,16 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>65.02</v>
+        <v>64.73999999999999</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3458,7 +3443,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3467,15 +3452,12 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>65.02</v>
+        <v>64.69</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E74" t="n">
-        <v>65</v>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
@@ -3489,21 +3471,24 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>64.87</v>
+        <v>64.64</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E75" t="n">
+        <v>65</v>
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
@@ -3517,16 +3502,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>64.75</v>
+        <v>64.56999999999999</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3548,16 +3533,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>64.73</v>
+        <v>64.56</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3579,16 +3564,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>64.56999999999999</v>
+        <v>64.52</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3610,16 +3595,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>64.52</v>
+        <v>64.47</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3636,21 +3621,25 @@
         </is>
       </c>
       <c r="H79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>64.47</v>
+        <v>64.44</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3667,25 +3656,21 @@
         </is>
       </c>
       <c r="H80" t="inlineStr"/>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
+      <c r="J80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>64.44</v>
+        <v>64.43000000000001</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3707,16 +3692,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>64.43000000000001</v>
+        <v>64.38</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3738,16 +3723,16 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>64.31</v>
+        <v>64.36</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3866,16 +3851,16 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>06 AI Compute Silicon / Programmable logic</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>64.06</v>
+        <v>63.92</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3897,16 +3882,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>UMAC</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Programmable logic</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>63.92</v>
+        <v>63.86</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3928,16 +3913,16 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>UMAC</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>63.86</v>
+        <v>63.84</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3959,24 +3944,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>63.84</v>
+        <v>63.78</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E90" t="n">
-        <v>80</v>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
@@ -3999,7 +3981,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>63.84</v>
+        <v>63.6</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -4018,21 +4000,24 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>63.78</v>
+        <v>63.57</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E92" t="n">
+        <v>80</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
@@ -4046,16 +4031,16 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>63.63</v>
+        <v>63.28</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -4077,16 +4062,16 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>63.28</v>
+        <v>63</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -4103,21 +4088,25 @@
         </is>
       </c>
       <c r="H94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>63</v>
+        <v>62.87</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -4134,11 +4123,7 @@
         </is>
       </c>
       <c r="H95" t="inlineStr"/>
-      <c r="J95" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
-        </is>
-      </c>
+      <c r="J95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4174,7 +4159,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SYM</t>
+          <t>6383.T</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4183,15 +4168,12 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>62.74</v>
+        <v>62.59</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E97" t="n">
-        <v>85</v>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
@@ -4205,21 +4187,24 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>6383.T</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>62.59</v>
+        <v>62.47</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E98" t="n">
+        <v>85</v>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
@@ -4233,16 +4218,16 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>SYM</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>62.47</v>
+        <v>62.38</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -4264,16 +4249,16 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>62.35</v>
+        <v>62.27</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -4295,16 +4280,16 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>62.27</v>
+        <v>62.25</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4326,16 +4311,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>62.25</v>
+        <v>62.13</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4478,16 +4463,16 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>61.47</v>
+        <v>61.52</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4509,16 +4494,16 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>61.42</v>
+        <v>61.47</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -4540,16 +4525,16 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>61.3</v>
+        <v>61.42</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -4571,16 +4556,16 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>61.05</v>
+        <v>61.01</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -4602,16 +4587,16 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>60.89</v>
+        <v>60.8</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -4633,16 +4618,16 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>60.86</v>
+        <v>60.77</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -4664,21 +4649,24 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2049.TW</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>60.8</v>
+        <v>60.6</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E113" t="n">
+        <v>99</v>
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
@@ -4692,16 +4680,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>MBLY</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>60.7</v>
+        <v>60.58</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4709,7 +4697,7 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
@@ -4723,16 +4711,16 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>RRX</t>
+          <t>SPCX</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>60.61</v>
+        <v>60.55</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -4740,7 +4728,7 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
@@ -4754,16 +4742,16 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>60.6</v>
+        <v>60.46</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -4771,7 +4759,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
@@ -4785,24 +4773,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>2049.TW</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>60.58</v>
+        <v>60.42</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E117" t="n">
-        <v>102</v>
       </c>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
@@ -4816,16 +4801,16 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>PRCT</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>60.46</v>
+        <v>60.27</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -4878,12 +4863,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>MBLY</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -4909,16 +4894,16 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>60.07</v>
+        <v>60.2</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -4940,16 +4925,16 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>SPCX</t>
+          <t>RRX</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>59.85</v>
+        <v>60.11</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -4971,16 +4956,16 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>RRC</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>59.83</v>
+        <v>59.69</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -5002,16 +4987,16 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>PRCT</t>
+          <t>AMKR</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>59.77</v>
+        <v>59.57</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -5033,16 +5018,16 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>RRC</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>59.69</v>
+        <v>59.39</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -5064,24 +5049,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>AMKR</t>
+          <t>6506.T</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>59.57</v>
+        <v>59.23</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E126" t="n">
-        <v>111</v>
       </c>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
@@ -5095,21 +5077,24 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>6506.T</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>10 Models, Software &amp; Applications / AI data layer</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>59.23</v>
+        <v>59.21</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E127" t="n">
+        <v>111</v>
       </c>
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
@@ -5123,16 +5108,16 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI data layer</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>59.21</v>
+        <v>59.1</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -5216,21 +5201,24 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>6481.T</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>10 Models, Software &amp; Applications / AI commerce</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>58.88</v>
+        <v>58.84</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E131" t="n">
+        <v>115</v>
       </c>
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
@@ -5244,24 +5232,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>KGX.DE</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI commerce</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>58.84</v>
+        <v>58.72</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E132" t="n">
-        <v>115</v>
       </c>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
@@ -5275,21 +5260,24 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>KGX.DE</t>
+          <t>UPST</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>58.72</v>
+        <v>58.68</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E133" t="n">
+        <v>116</v>
       </c>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
@@ -5303,24 +5291,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>UPST</t>
+          <t>6481.T</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>58.68</v>
+        <v>58.5</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E134" t="n">
-        <v>116</v>
       </c>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
@@ -5334,16 +5319,16 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>58.48</v>
+        <v>58.4</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -5365,16 +5350,16 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>58.4</v>
+        <v>58.33</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
@@ -5396,16 +5381,16 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>58.33</v>
+        <v>58.11</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
@@ -5427,16 +5412,16 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>58.18</v>
+        <v>58.01</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
@@ -5458,16 +5443,16 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>ASX</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>58.04</v>
+        <v>57.89</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
@@ -5489,7 +5474,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -5498,7 +5483,7 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>58.01</v>
+        <v>57.82</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
@@ -5520,16 +5505,16 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>ONDS</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>57.95</v>
+        <v>57.81</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -5551,16 +5536,16 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>WYFI</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>57.89</v>
+        <v>57.67</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
@@ -5582,16 +5567,16 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>WYFI</t>
+          <t>ASX</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>57.67</v>
+        <v>57.61</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -5613,21 +5598,24 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>DRO.AX</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>57.49</v>
+        <v>57.57</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E144" t="n">
+        <v>126</v>
       </c>
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
@@ -5641,24 +5629,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>CARR</t>
+          <t>DRO.AX</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>57.44</v>
+        <v>57.49</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E145" t="n">
-        <v>126</v>
       </c>
       <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
@@ -5672,16 +5657,16 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>ONDS</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>57.32</v>
+        <v>57.45</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
@@ -5796,16 +5781,16 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>TKR</t>
+          <t>AVAV</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>56.86</v>
+        <v>56.81</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
@@ -5827,16 +5812,16 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>AVAV</t>
+          <t>CARR</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>56.81</v>
+        <v>56.71</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
@@ -5858,16 +5843,16 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>HIVE</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>56.71</v>
+        <v>56.62</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -5889,16 +5874,16 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>HIVE</t>
+          <t>PPL</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>56.62</v>
+        <v>56.52</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -5920,16 +5905,16 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>TKR</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>56.21</v>
+        <v>56.48</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -5982,16 +5967,16 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>PPL</t>
+          <t>PSIX</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>56.02</v>
+        <v>55.93</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
@@ -6013,16 +5998,16 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>55.95</v>
+        <v>55.71</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
@@ -6044,24 +6029,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>PSIX</t>
+          <t>6324.T</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>55.93</v>
+        <v>55.69</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E158" t="n">
-        <v>139</v>
       </c>
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
@@ -6084,7 +6066,7 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>55.86</v>
+        <v>55.69</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
@@ -6092,7 +6074,7 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
@@ -6106,21 +6088,24 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>6324.T</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>55.69</v>
+        <v>55.45</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E160" t="n">
+        <v>140</v>
       </c>
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
@@ -6134,24 +6119,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>2590.HK</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>55.29</v>
+        <v>55.27</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E161" t="n">
-        <v>141</v>
       </c>
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
@@ -6165,21 +6147,24 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2590.HK</t>
+          <t>BW</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>55.27</v>
+        <v>55.17</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E162" t="n">
+        <v>141</v>
       </c>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
@@ -6193,16 +6178,16 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>BW</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>55.17</v>
+        <v>55.14</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
@@ -6220,37 +6205,6 @@
       </c>
       <c r="H163" t="inlineStr"/>
       <c r="J163" t="inlineStr"/>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>AEP</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
-        </is>
-      </c>
-      <c r="C164" t="n">
-        <v>55.14</v>
-      </c>
-      <c r="D164" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E164" t="n">
-        <v>143</v>
-      </c>
-      <c r="F164" t="inlineStr"/>
-      <c r="G164" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H164" t="inlineStr"/>
-      <c r="J164" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
daily-watch 2026-10-26: FIX/WDC/LRCX re-scored; EME+VRT exit, LRCX enters; ticket HELD (#205)
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-18 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-10-26 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J164"/>
+  <dimension ref="A1:J163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1068,7 +1068,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-10-18, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-10-26, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1127,20 +1127,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>84.39</v>
+        <v>85.83</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓✓✓</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1158,23 +1158,27 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J3" t="inlineStr"/>
+        <v>6.25</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>82.38</v>
+        <v>83.87</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1196,23 +1200,23 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>81.90000000000001</v>
+        <v>82.38</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1234,27 +1238,23 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
-        </is>
-      </c>
+        <v>6.25</v>
+      </c>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>81.58</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1276,27 +1276,27 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
+          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>81.44</v>
+        <v>81.58</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1318,18 +1318,18 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1360,23 +1360,23 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>79.53</v>
+        <v>79.79000000000001</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1398,23 +1398,23 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>79.40000000000001</v>
+        <v>79.53</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1436,23 +1436,23 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06 Silicon - Memory</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>78.77</v>
+        <v>79.15000000000001</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1474,23 +1474,23 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>06 Silicon - Memory</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>76.40000000000001</v>
+        <v>78.39</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1512,23 +1512,23 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>75.8</v>
+        <v>76.27</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1550,23 +1550,23 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RDDT</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>75.53</v>
+        <v>75.8</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1588,51 +1588,61 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>6861.T</t>
+          <t>RDDT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>74.28</v>
+        <v>75.53</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
+      <c r="E15" t="n">
+        <v>13</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>6.25</v>
+      </c>
       <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GMED</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>73.92</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1640,7 +1650,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1654,61 +1664,51 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>5.88</v>
+        <v>6.25</v>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>6861.T</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>73.91</v>
+        <v>74.28</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E17" t="n">
-        <v>14</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="n">
-        <v>5.88</v>
-      </c>
       <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>73.75</v>
+        <v>74.03</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1720,58 +1720,71 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>ENTRY DEFERRED (rank 15, score 73.8; entry hold until 2026-11-15: San Diego County enforcement action filed 2026-10-05 (People v. AppLovin, seeks an injunction on data collection) and securities class action Talbot v. AppLovin, 3:26-cv-10584 (N.D. Cal., filed 2026-09-16); growth decelerating with Q3 uplift untested)</t>
+          <t>ENTER (rank 15, score 74.0)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
+      <c r="I18" t="n">
+        <v>6.25</v>
+      </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>GMED</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>73.51000000000001</v>
+        <v>73.92</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>16</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
+      <c r="I19" t="n">
+        <v>6.25</v>
+      </c>
       <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>73.48</v>
+        <v>73.75</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1779,75 +1792,58 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>16</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="n">
-        <v>5.88</v>
-      </c>
       <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>03 DC Infrastructure</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>73.25</v>
+        <v>73.51000000000001</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E21" t="n">
-        <v>17</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="n">
-        <v>5.88</v>
-      </c>
       <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>73.17</v>
+        <v>73.27</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1857,25 +1853,14 @@
       <c r="E22" t="n">
         <v>18</v>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1911,16 +1896,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>72.65000000000001</v>
+        <v>72.87</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1937,21 +1922,25 @@
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>03 DC Infrastructure</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>72.38</v>
+        <v>72.75</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1973,16 +1962,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>72.25</v>
+        <v>72.38</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1992,11 +1981,7 @@
       <c r="E26" t="n">
         <v>22</v>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>EXIT (pending since 2026-10-11, confirmed)</t>
-        </is>
-      </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>N</t>
@@ -2008,16 +1993,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>72.23999999999999</v>
+        <v>72.25</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2070,16 +2055,16 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>71.81999999999999</v>
+        <v>71.86</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2101,16 +2086,16 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>71.81</v>
+        <v>71.58</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2132,16 +2117,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>71.58</v>
+        <v>71.45</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2163,21 +2148,24 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BSL.DE</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>70.95999999999999</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
+      </c>
+      <c r="E32" t="n">
+        <v>28</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
@@ -2191,24 +2179,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>BSL.DE</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>70.23</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
-      </c>
-      <c r="E33" t="n">
-        <v>28</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
@@ -2222,16 +2207,16 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>70.19</v>
+        <v>70.68000000000001</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2253,16 +2238,16 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>69.95999999999999</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2284,24 +2269,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>HTHIY</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>69.53</v>
+        <v>69.17</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E36" t="n">
-        <v>31</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
@@ -2315,12 +2297,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>HTHIY</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -2331,6 +2313,9 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="E37" t="n">
+        <v>31</v>
+      </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
@@ -2374,16 +2359,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>CGNX</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>68.89</v>
+        <v>68.88</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2405,16 +2390,16 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CGNX</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>68.88</v>
+        <v>68.86</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2436,16 +2421,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>68.86</v>
+        <v>68.45999999999999</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2467,16 +2452,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>68.73</v>
+        <v>68.45999999999999</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2498,16 +2483,16 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>68.67</v>
+        <v>68.31999999999999</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2524,21 +2509,25 @@
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>NTAP</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>68.45999999999999</v>
+        <v>68.31</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2560,16 +2549,16 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>NOVT</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>68.31999999999999</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2586,25 +2575,21 @@
         </is>
       </c>
       <c r="H45" t="inlineStr"/>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
-        </is>
-      </c>
+      <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>NOVT</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>68.12</v>
+        <v>68</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2626,24 +2611,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>6268.T</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>68.11</v>
+        <v>67.98</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E47" t="n">
-        <v>41</v>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
@@ -2657,16 +2639,16 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>68</v>
+        <v>67.95</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2674,7 +2656,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
@@ -2688,21 +2670,24 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>6268.T</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>67.98</v>
+        <v>67.73</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E49" t="n">
+        <v>42</v>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
@@ -2716,16 +2701,16 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>67.90000000000001</v>
+        <v>67.7</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2747,16 +2732,16 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>67.7</v>
+        <v>67.42</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2773,21 +2758,25 @@
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>67.42</v>
+        <v>67.22</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -2804,30 +2793,29 @@
         </is>
       </c>
       <c r="H52" t="inlineStr"/>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
-        </is>
-      </c>
+      <c r="J52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>6954.T</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>67.33</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E53" t="n">
+        <v>46</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
@@ -2841,16 +2829,16 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>MKSI</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>67.31</v>
+        <v>67</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2858,7 +2846,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
@@ -2872,16 +2860,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>67.22</v>
+        <v>67</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2889,7 +2877,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
@@ -2903,7 +2891,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2912,7 +2900,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>67.15000000000001</v>
+        <v>66.93000000000001</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -2920,7 +2908,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
@@ -2934,24 +2922,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MKSI</t>
+          <t>6954.T</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>67.12</v>
+        <v>66.83</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E57" t="n">
-        <v>49</v>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
@@ -2965,16 +2950,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>WDAY</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>67</v>
+        <v>66.73</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2996,16 +2981,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>66.89</v>
+        <v>66.72</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3027,16 +3012,16 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>66.72</v>
+        <v>66.27</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3058,21 +3043,24 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>AUTO.OL</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>66.51000000000001</v>
+        <v>66.20999999999999</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E61" t="n">
+        <v>53</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
@@ -3086,24 +3074,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>AUTO.OL</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>66.02</v>
+        <v>66.13</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E62" t="n">
-        <v>53</v>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
@@ -3117,16 +3102,16 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>65.97</v>
+        <v>66.02</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3179,16 +3164,16 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>65.73</v>
+        <v>65.67</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3210,16 +3195,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>65.73</v>
+        <v>65.61</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3241,16 +3226,16 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>65.48999999999999</v>
+        <v>65.31</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3272,16 +3257,16 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>OUST</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>65.38</v>
+        <v>65.20999999999999</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3303,16 +3288,16 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>65.29000000000001</v>
+        <v>65.04000000000001</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3334,16 +3319,16 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>65.25</v>
+        <v>65.02</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3365,16 +3350,16 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>OUST</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>65.20999999999999</v>
+        <v>64.88</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3396,16 +3381,16 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>65.04000000000001</v>
+        <v>64.75</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3427,16 +3412,16 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>65.02</v>
+        <v>64.73999999999999</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3458,7 +3443,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3467,15 +3452,12 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>65.02</v>
+        <v>64.69</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E74" t="n">
-        <v>65</v>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
@@ -3489,21 +3471,24 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>64.87</v>
+        <v>64.64</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E75" t="n">
+        <v>65</v>
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
@@ -3517,16 +3502,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>64.75</v>
+        <v>64.56999999999999</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3548,16 +3533,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>64.73</v>
+        <v>64.56</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3579,16 +3564,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>64.56999999999999</v>
+        <v>64.52</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3610,16 +3595,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>64.52</v>
+        <v>64.47</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3636,21 +3621,25 @@
         </is>
       </c>
       <c r="H79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>64.47</v>
+        <v>64.44</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3667,25 +3656,21 @@
         </is>
       </c>
       <c r="H80" t="inlineStr"/>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
+      <c r="J80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>64.44</v>
+        <v>64.43000000000001</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3707,16 +3692,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>64.43000000000001</v>
+        <v>64.38</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3738,16 +3723,16 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>64.31</v>
+        <v>64.36</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3866,16 +3851,16 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>06 AI Compute Silicon / Programmable logic</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>64.06</v>
+        <v>63.92</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3897,16 +3882,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>UMAC</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Programmable logic</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>63.92</v>
+        <v>63.86</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3928,16 +3913,16 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>UMAC</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>63.86</v>
+        <v>63.84</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3959,24 +3944,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>63.84</v>
+        <v>63.78</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E90" t="n">
-        <v>80</v>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
@@ -3999,7 +3981,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>63.84</v>
+        <v>63.6</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -4018,21 +4000,24 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>63.78</v>
+        <v>63.57</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E92" t="n">
+        <v>80</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
@@ -4046,16 +4031,16 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>63.63</v>
+        <v>63.28</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -4077,16 +4062,16 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>63.28</v>
+        <v>63</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -4103,21 +4088,25 @@
         </is>
       </c>
       <c r="H94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>63</v>
+        <v>62.87</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -4134,11 +4123,7 @@
         </is>
       </c>
       <c r="H95" t="inlineStr"/>
-      <c r="J95" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
-        </is>
-      </c>
+      <c r="J95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4174,7 +4159,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SYM</t>
+          <t>6383.T</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4183,15 +4168,12 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>62.74</v>
+        <v>62.59</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E97" t="n">
-        <v>85</v>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
@@ -4205,21 +4187,24 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>6383.T</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>62.59</v>
+        <v>62.47</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E98" t="n">
+        <v>85</v>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
@@ -4233,16 +4218,16 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>SYM</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>62.47</v>
+        <v>62.38</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -4264,16 +4249,16 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>62.35</v>
+        <v>62.27</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -4295,16 +4280,16 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>62.27</v>
+        <v>62.25</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4326,16 +4311,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>62.25</v>
+        <v>62.13</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4478,16 +4463,16 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>61.47</v>
+        <v>61.52</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4509,16 +4494,16 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>61.42</v>
+        <v>61.47</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -4540,16 +4525,16 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>61.3</v>
+        <v>61.42</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -4571,16 +4556,16 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>61.05</v>
+        <v>61.01</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -4602,16 +4587,16 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>60.89</v>
+        <v>60.8</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -4633,16 +4618,16 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>60.86</v>
+        <v>60.77</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -4664,21 +4649,24 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2049.TW</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>60.8</v>
+        <v>60.6</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E113" t="n">
+        <v>99</v>
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
@@ -4692,16 +4680,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>MBLY</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>60.7</v>
+        <v>60.58</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4709,7 +4697,7 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
@@ -4723,16 +4711,16 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>RRX</t>
+          <t>SPCX</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>60.61</v>
+        <v>60.55</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -4740,7 +4728,7 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
@@ -4754,16 +4742,16 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>60.6</v>
+        <v>60.46</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -4771,7 +4759,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
@@ -4785,24 +4773,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>2049.TW</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>60.58</v>
+        <v>60.42</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E117" t="n">
-        <v>102</v>
       </c>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
@@ -4816,16 +4801,16 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>PRCT</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>60.46</v>
+        <v>60.27</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -4878,12 +4863,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>MBLY</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -4909,16 +4894,16 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>60.07</v>
+        <v>60.2</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -4940,16 +4925,16 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>SPCX</t>
+          <t>RRX</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>59.85</v>
+        <v>60.11</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -4971,16 +4956,16 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>RRC</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>59.83</v>
+        <v>59.69</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -5002,16 +4987,16 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>PRCT</t>
+          <t>AMKR</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>59.77</v>
+        <v>59.57</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -5033,16 +5018,16 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>RRC</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>59.69</v>
+        <v>59.39</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -5064,24 +5049,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>AMKR</t>
+          <t>6506.T</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>59.57</v>
+        <v>59.23</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E126" t="n">
-        <v>111</v>
       </c>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
@@ -5095,21 +5077,24 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>6506.T</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>10 Models, Software &amp; Applications / AI data layer</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>59.23</v>
+        <v>59.21</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E127" t="n">
+        <v>111</v>
       </c>
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
@@ -5123,16 +5108,16 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI data layer</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>59.21</v>
+        <v>59.1</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -5216,21 +5201,24 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>6481.T</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>10 Models, Software &amp; Applications / AI commerce</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>58.88</v>
+        <v>58.84</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E131" t="n">
+        <v>115</v>
       </c>
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
@@ -5244,24 +5232,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>KGX.DE</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI commerce</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>58.84</v>
+        <v>58.72</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E132" t="n">
-        <v>115</v>
       </c>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
@@ -5275,21 +5260,24 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>KGX.DE</t>
+          <t>UPST</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>58.72</v>
+        <v>58.68</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E133" t="n">
+        <v>116</v>
       </c>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
@@ -5303,24 +5291,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>UPST</t>
+          <t>6481.T</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>58.68</v>
+        <v>58.5</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E134" t="n">
-        <v>116</v>
       </c>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
@@ -5334,16 +5319,16 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>58.48</v>
+        <v>58.4</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -5365,16 +5350,16 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>58.4</v>
+        <v>58.33</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
@@ -5396,16 +5381,16 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>58.33</v>
+        <v>58.11</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
@@ -5427,16 +5412,16 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>58.18</v>
+        <v>58.01</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
@@ -5458,16 +5443,16 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>ASX</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>58.04</v>
+        <v>57.89</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
@@ -5489,7 +5474,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -5498,7 +5483,7 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>58.01</v>
+        <v>57.82</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
@@ -5520,16 +5505,16 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>ONDS</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>57.95</v>
+        <v>57.81</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -5551,16 +5536,16 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>WYFI</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>57.89</v>
+        <v>57.67</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
@@ -5582,16 +5567,16 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>WYFI</t>
+          <t>ASX</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>57.67</v>
+        <v>57.61</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -5613,21 +5598,24 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>DRO.AX</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>57.49</v>
+        <v>57.57</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E144" t="n">
+        <v>126</v>
       </c>
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
@@ -5641,24 +5629,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>CARR</t>
+          <t>DRO.AX</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>57.44</v>
+        <v>57.49</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E145" t="n">
-        <v>126</v>
       </c>
       <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
@@ -5672,16 +5657,16 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>ONDS</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>57.32</v>
+        <v>57.45</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
@@ -5796,16 +5781,16 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>TKR</t>
+          <t>AVAV</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>56.86</v>
+        <v>56.81</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
@@ -5827,16 +5812,16 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>AVAV</t>
+          <t>CARR</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>56.81</v>
+        <v>56.71</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
@@ -5858,16 +5843,16 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>HIVE</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>56.71</v>
+        <v>56.62</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -5889,16 +5874,16 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>HIVE</t>
+          <t>PPL</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>56.62</v>
+        <v>56.52</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -5920,16 +5905,16 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>TKR</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>56.21</v>
+        <v>56.48</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -5982,16 +5967,16 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>PPL</t>
+          <t>PSIX</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>56.02</v>
+        <v>55.93</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
@@ -6013,16 +5998,16 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>55.95</v>
+        <v>55.71</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
@@ -6044,24 +6029,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>PSIX</t>
+          <t>6324.T</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>55.93</v>
+        <v>55.69</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E158" t="n">
-        <v>139</v>
       </c>
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
@@ -6084,7 +6066,7 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>55.86</v>
+        <v>55.69</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
@@ -6092,7 +6074,7 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
@@ -6106,21 +6088,24 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>6324.T</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>55.69</v>
+        <v>55.45</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E160" t="n">
+        <v>140</v>
       </c>
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
@@ -6134,24 +6119,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>2590.HK</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>55.29</v>
+        <v>55.27</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E161" t="n">
-        <v>141</v>
       </c>
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
@@ -6165,21 +6147,24 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2590.HK</t>
+          <t>BW</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>55.27</v>
+        <v>55.17</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E162" t="n">
+        <v>141</v>
       </c>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
@@ -6193,16 +6178,16 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>BW</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>55.17</v>
+        <v>55.14</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
@@ -6220,37 +6205,6 @@
       </c>
       <c r="H163" t="inlineStr"/>
       <c r="J163" t="inlineStr"/>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>AEP</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
-        </is>
-      </c>
-      <c r="C164" t="n">
-        <v>55.14</v>
-      </c>
-      <c r="D164" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E164" t="n">
-        <v>143</v>
-      </c>
-      <c r="F164" t="inlineStr"/>
-      <c r="G164" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H164" t="inlineStr"/>
-      <c r="J164" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
daily-watch 2026-10-29: EME beat re-scored to rank 15 and enters (ticket HELD); SNDK/RDDT/AMZN briefed; META equity raise; RDDT R5 proposal
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-26 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-10-29 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-10-26, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-10-29, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>85.83</v>
+        <v>85.53</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J4" t="inlineStr"/>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J5" t="inlineStr"/>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J13" t="inlineStr"/>
     </row>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J15" t="inlineStr"/>
     </row>
@@ -1664,89 +1664,93 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>6861.T</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>74.28</v>
+        <v>74.48</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
+      <c r="E17" t="n">
+        <v>15</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>ENTER (rank 15, score 74.5)</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>6861.T</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>74.03</v>
+        <v>74.28</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>15</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>ENTER (rank 15, score 74.0)</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="n">
-        <v>6.25</v>
-      </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GMED</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>73.92</v>
+        <v>74.03</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1768,23 +1772,23 @@
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>GMED</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>73.75</v>
+        <v>73.92</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1794,33 +1798,43 @@
       <c r="E20" t="n">
         <v>17</v>
       </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
+      <c r="I20" t="n">
+        <v>5.88</v>
+      </c>
       <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>73.51000000000001</v>
+        <v>73.75</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
+      </c>
+      <c r="E21" t="n">
+        <v>18</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
@@ -1834,24 +1848,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>73.27</v>
+        <v>73.51000000000001</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
-      </c>
-      <c r="E22" t="n">
-        <v>18</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
@@ -1865,16 +1876,16 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>72.98999999999999</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1896,16 +1907,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>72.87</v>
+        <v>72.98999999999999</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1922,11 +1933,7 @@
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1962,16 +1969,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>72.38</v>
+        <v>72.64</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1993,16 +2000,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>72.25</v>
+        <v>72.38</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2024,7 +2031,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2033,7 +2040,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>71.88</v>
+        <v>72.25</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2055,16 +2062,16 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>71.86</v>
+        <v>71.88</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2891,24 +2898,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>6954.T</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>66.93000000000001</v>
+        <v>66.83</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E56" t="n">
-        <v>49</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
@@ -2922,21 +2926,24 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>6954.T</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>66.83</v>
+        <v>66.73</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E57" t="n">
+        <v>49</v>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
@@ -2950,16 +2957,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>66.73</v>
+        <v>66.72</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2981,16 +2988,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>66.72</v>
+        <v>66.65000000000001</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3471,16 +3478,16 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>64.64</v>
+        <v>64.56999999999999</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3502,16 +3509,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>64.56999999999999</v>
+        <v>64.56</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3533,16 +3540,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>64.56</v>
+        <v>64.52</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3564,16 +3571,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>64.52</v>
+        <v>64.47</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3590,21 +3597,25 @@
         </is>
       </c>
       <c r="H78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>64.47</v>
+        <v>64.44</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3621,25 +3632,21 @@
         </is>
       </c>
       <c r="H79" t="inlineStr"/>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
+      <c r="J79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>64.44</v>
+        <v>64.43000000000001</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3661,16 +3668,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>64.43000000000001</v>
+        <v>64.38</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3692,16 +3699,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>64.38</v>
+        <v>64.36</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3723,16 +3730,16 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>64.36</v>
+        <v>64.34</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
daily-watch 2026-10-29: EME beat re-scored to rank 15 and enters (ticket HELD); SNDK/RDDT/AMZN briefed; META equity raise; RDDT R5 proposal (#225)
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-26 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-10-29 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-10-26, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-10-29, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>85.83</v>
+        <v>85.53</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J4" t="inlineStr"/>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J5" t="inlineStr"/>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J13" t="inlineStr"/>
     </row>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J15" t="inlineStr"/>
     </row>
@@ -1664,89 +1664,93 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>6861.T</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>74.28</v>
+        <v>74.48</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
+      <c r="E17" t="n">
+        <v>15</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>ENTER (rank 15, score 74.5)</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>6861.T</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>74.03</v>
+        <v>74.28</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>15</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>ENTER (rank 15, score 74.0)</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="n">
-        <v>6.25</v>
-      </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GMED</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>73.92</v>
+        <v>74.03</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1768,23 +1772,23 @@
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
-        <v>6.25</v>
+        <v>5.88</v>
       </c>
       <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>GMED</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>73.75</v>
+        <v>73.92</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1794,33 +1798,43 @@
       <c r="E20" t="n">
         <v>17</v>
       </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
+      <c r="I20" t="n">
+        <v>5.88</v>
+      </c>
       <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>73.51000000000001</v>
+        <v>73.75</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
+      </c>
+      <c r="E21" t="n">
+        <v>18</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
@@ -1834,24 +1848,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>73.27</v>
+        <v>73.51000000000001</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
-      </c>
-      <c r="E22" t="n">
-        <v>18</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
@@ -1865,16 +1876,16 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>72.98999999999999</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1896,16 +1907,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>72.87</v>
+        <v>72.98999999999999</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1922,11 +1933,7 @@
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1962,16 +1969,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>72.38</v>
+        <v>72.64</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1993,16 +2000,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>72.25</v>
+        <v>72.38</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2024,7 +2031,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2033,7 +2040,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>71.88</v>
+        <v>72.25</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2055,16 +2062,16 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>71.86</v>
+        <v>71.88</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2891,24 +2898,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>6954.T</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>66.93000000000001</v>
+        <v>66.83</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E56" t="n">
-        <v>49</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
@@ -2922,21 +2926,24 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>6954.T</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>66.83</v>
+        <v>66.73</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E57" t="n">
+        <v>49</v>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
@@ -2950,16 +2957,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>66.73</v>
+        <v>66.72</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2981,16 +2988,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>66.72</v>
+        <v>66.65000000000001</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3471,16 +3478,16 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>64.64</v>
+        <v>64.56999999999999</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3502,16 +3509,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>64.56999999999999</v>
+        <v>64.56</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3533,16 +3540,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>64.56</v>
+        <v>64.52</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3564,16 +3571,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>64.52</v>
+        <v>64.47</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3590,21 +3597,25 @@
         </is>
       </c>
       <c r="H78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>64.47</v>
+        <v>64.44</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3621,25 +3632,21 @@
         </is>
       </c>
       <c r="H79" t="inlineStr"/>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
+      <c r="J79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>64.44</v>
+        <v>64.43000000000001</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3661,16 +3668,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>64.43000000000001</v>
+        <v>64.38</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3692,16 +3699,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>64.38</v>
+        <v>64.36</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3723,16 +3730,16 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>64.36</v>
+        <v>64.34</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
rescore 2026-10-30: refresh prices and scores for all names
Full objective, 50DMA and reverse-DCF refresh after 179 names had gone
stale since 2026-10-11. Model adds VRT and ASML; MU moves to the top
tier; WDC and LRCX exit clocks start.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-29 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-10-30 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J163"/>
+  <dimension ref="A1:J166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1068,7 +1068,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-10-29, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-10-30, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1127,16 +1127,16 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>06 Silicon - Memory</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>85.53</v>
+        <v>88.7</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1158,31 +1158,27 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
-        </is>
-      </c>
+        <v>5.26</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>83.87</v>
+        <v>85.27</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓✓✓</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1200,23 +1196,27 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J4" t="inlineStr"/>
+        <v>5.26</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>82.38</v>
+        <v>83.64</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1238,23 +1238,23 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>81.90000000000001</v>
+        <v>82.95999999999999</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1276,27 +1276,23 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
-        </is>
-      </c>
+        <v>5.26</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>81.58</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1318,27 +1314,27 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
+          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>79.79000000000001</v>
+        <v>82.20999999999999</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1360,9 +1356,13 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J8" t="inlineStr"/>
+        <v>5.26</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>79.79000000000001</v>
+        <v>80.79000000000001</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1398,23 +1398,23 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>79.53</v>
+        <v>80.43000000000001</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1436,23 +1436,23 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>79.15000000000001</v>
+        <v>79.12</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1474,23 +1474,23 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06 Silicon - Memory</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>78.39</v>
+        <v>78.73</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1512,23 +1512,23 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>RDDT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>76.27</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1550,23 +1550,23 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>75.8</v>
+        <v>76.02</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1588,23 +1588,27 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J14" t="inlineStr"/>
+        <v>5.26</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RDDT</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>75.53</v>
+        <v>75.79000000000001</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1626,23 +1630,23 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>74.79000000000001</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1664,23 +1668,23 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>74.48</v>
+        <v>74.73999999999999</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1692,7 +1696,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ENTER (rank 15, score 74.5)</t>
+          <t>ENTER (rank 15, score 74.7)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1702,55 +1706,61 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+        <v>5.26</v>
+      </c>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>6861.T</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>03 DC Infrastructure</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>74.28</v>
+        <v>74.5</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="E18" t="n">
+        <v>16</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
+      <c r="I18" t="n">
+        <v>5.26</v>
+      </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>74.03</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1758,75 +1768,58 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>16</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="n">
-        <v>5.88</v>
-      </c>
       <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GMED</t>
+          <t>6861.T</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>73.92</v>
+        <v>73.73</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E20" t="n">
-        <v>17</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="n">
-        <v>5.88</v>
-      </c>
       <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>GMED</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>73.75</v>
+        <v>73.42</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1836,33 +1829,43 @@
       <c r="E21" t="n">
         <v>18</v>
       </c>
-      <c r="F21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
+      <c r="I21" t="n">
+        <v>5.26</v>
+      </c>
       <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>73.51000000000001</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
+      </c>
+      <c r="E22" t="n">
+        <v>19</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
@@ -1876,16 +1879,16 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>73.40000000000001</v>
+        <v>73.16</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1893,7 +1896,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
@@ -1907,16 +1910,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>72.98999999999999</v>
+        <v>72.89</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1924,26 +1927,33 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>20</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>EXIT PENDING (rank 21 &gt; exit rank 18, since 2026-10-30)</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
+      <c r="I24" t="n">
+        <v>5.26</v>
+      </c>
       <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>03 DC Infrastructure</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1955,7 +1965,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
@@ -1969,16 +1979,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>72.64</v>
+        <v>72.70999999999999</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1986,7 +1996,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
@@ -2000,24 +2010,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>72.38</v>
+        <v>72.66</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
-      </c>
-      <c r="E27" t="n">
-        <v>23</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
@@ -2031,16 +2038,16 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>72.25</v>
+        <v>72.28</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2050,28 +2057,35 @@
       <c r="E28" t="n">
         <v>24</v>
       </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>EXIT PENDING (rank 24 &gt; exit rank 18, since 2026-10-30)</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
+      <c r="I28" t="n">
+        <v>5.26</v>
+      </c>
       <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>71.88</v>
+        <v>72.08</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2102,7 +2116,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>71.58</v>
+        <v>72.08</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2124,16 +2138,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>71.45</v>
+        <v>71.48</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2155,16 +2169,16 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>71.09999999999999</v>
+        <v>71.17</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2186,21 +2200,24 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BSL.DE</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>70.95999999999999</v>
+        <v>70.64</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
+      </c>
+      <c r="E33" t="n">
+        <v>29</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
@@ -2214,24 +2231,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>6954.T</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>70.68000000000001</v>
+        <v>70.63</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
-      </c>
-      <c r="E34" t="n">
-        <v>29</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
@@ -2245,7 +2259,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2254,11 +2268,11 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>69.26000000000001</v>
+        <v>70.55</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -2276,20 +2290,20 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>HTHIY</t>
+          <t>BSL.DE</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>69.17</v>
+        <v>70.36</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -2304,7 +2318,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2313,11 +2327,11 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>69.17</v>
+        <v>70.11</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -2335,16 +2349,16 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>69.15000000000001</v>
+        <v>69.91</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2366,16 +2380,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CGNX</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>68.88</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2397,16 +2411,16 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>68.86</v>
+        <v>69.69</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2428,16 +2442,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>68.45999999999999</v>
+        <v>69.45</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2459,16 +2473,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>68.45999999999999</v>
+        <v>69.44</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2490,24 +2504,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>HTHIY</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>68.31999999999999</v>
+        <v>69.33</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E43" t="n">
-        <v>37</v>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
@@ -2516,25 +2527,21 @@
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
-        </is>
-      </c>
+      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>CGNX</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>68.31</v>
+        <v>69.15000000000001</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2542,7 +2549,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
@@ -2556,16 +2563,16 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>NOVT</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>68.20999999999999</v>
+        <v>69.11</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2573,7 +2580,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
@@ -2587,16 +2594,16 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>68</v>
+        <v>68.77</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2604,7 +2611,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
@@ -2618,16 +2625,16 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>6268.T</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>67.98</v>
+        <v>68.73</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2646,16 +2653,16 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>67.95</v>
+        <v>68.43000000000001</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2663,7 +2670,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
@@ -2677,16 +2684,16 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>NTAP</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>67.73</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2694,7 +2701,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
@@ -2708,16 +2715,16 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>67.7</v>
+        <v>67.98999999999999</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2725,7 +2732,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
@@ -2739,16 +2746,16 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>67.42</v>
+        <v>67.81999999999999</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2756,7 +2763,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
@@ -2765,25 +2772,21 @@
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
-        </is>
-      </c>
+      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>67.22</v>
+        <v>67.73999999999999</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -2791,7 +2794,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
@@ -2805,16 +2808,16 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>NOVT</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>67.15000000000001</v>
+        <v>67.69</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -2822,7 +2825,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
@@ -2836,16 +2839,16 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MKSI</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>67</v>
+        <v>67.56999999999999</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2853,7 +2856,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
@@ -2867,16 +2870,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>WDAY</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
+          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>67</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2884,7 +2887,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
@@ -2898,21 +2901,24 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>6954.T</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>66.83</v>
+        <v>67.51000000000001</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E56" t="n">
+        <v>48</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
@@ -2921,21 +2927,25 @@
         </is>
       </c>
       <c r="H56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>66.73</v>
+        <v>67.34</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -2952,21 +2962,25 @@
         </is>
       </c>
       <c r="H57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>10 Models, Software &amp; Applications / Consumer fintech (AI adopter)</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>66.72</v>
+        <v>67.23999999999999</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2988,16 +3002,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>66.65000000000001</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3019,16 +3033,16 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>66.27</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3050,16 +3064,16 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>66.20999999999999</v>
+        <v>67.14</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -3081,16 +3095,16 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>AUTO.OL</t>
+          <t>6268.T</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>66.13</v>
+        <v>66.97</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3109,16 +3123,16 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>66.02</v>
+        <v>66.77</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3140,16 +3154,16 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>65.95999999999999</v>
+        <v>66.66</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3171,16 +3185,16 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>MKSI</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>65.67</v>
+        <v>66.36</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3202,16 +3216,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>65.61</v>
+        <v>66.31999999999999</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3233,16 +3247,16 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>65.31</v>
+        <v>66.3</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3264,24 +3278,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>OUST</t>
+          <t>AUTO.OL</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>65.20999999999999</v>
+        <v>66.27</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E68" t="n">
-        <v>59</v>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
@@ -3295,16 +3306,16 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>65.04000000000001</v>
+        <v>66.2</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3312,7 +3323,7 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
@@ -3326,16 +3337,16 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>65.02</v>
+        <v>65.95999999999999</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3343,7 +3354,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
@@ -3357,16 +3368,16 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>64.88</v>
+        <v>65.95</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3374,7 +3385,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
@@ -3388,16 +3399,16 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>64.75</v>
+        <v>65.79000000000001</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3405,7 +3416,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
@@ -3419,16 +3430,16 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>64.73999999999999</v>
+        <v>65.73</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3436,7 +3447,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
@@ -3450,21 +3461,24 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>64.69</v>
+        <v>65.45</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E74" t="n">
+        <v>64</v>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
@@ -3478,16 +3492,16 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>64.56999999999999</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3509,16 +3523,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>64.56</v>
+        <v>65.27</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3540,16 +3554,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>64.52</v>
+        <v>65.26000000000001</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3571,16 +3585,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>64.47</v>
+        <v>65.06999999999999</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3597,25 +3611,21 @@
         </is>
       </c>
       <c r="H78" t="inlineStr"/>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
+      <c r="J78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>64.44</v>
+        <v>65.04000000000001</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3637,16 +3647,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>64.43000000000001</v>
+        <v>65.02</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3668,16 +3678,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>OUST</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>64.38</v>
+        <v>64.97</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3699,16 +3709,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>64.36</v>
+        <v>64.88</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3730,24 +3740,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>64.34</v>
+        <v>64.5</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E83" t="n">
-        <v>73</v>
       </c>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
@@ -3761,16 +3768,16 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>GNRC</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>64.28</v>
+        <v>64.37</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -3778,7 +3785,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
@@ -3792,16 +3799,16 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>64.15000000000001</v>
+        <v>64.34999999999999</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -3809,7 +3816,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
@@ -3818,25 +3825,21 @@
         </is>
       </c>
       <c r="H85" t="inlineStr"/>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
-        </is>
-      </c>
+      <c r="J85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>PLAB</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>64.08</v>
+        <v>64.33</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3844,7 +3847,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
@@ -3858,16 +3861,16 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Programmable logic</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>63.92</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3875,7 +3878,7 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
@@ -3889,16 +3892,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>UMAC</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>63.86</v>
+        <v>64.27</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3906,7 +3909,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
@@ -3915,21 +3918,25 @@
         </is>
       </c>
       <c r="H88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>PLAB</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>63.84</v>
+        <v>64.17</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3937,7 +3944,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
@@ -3951,21 +3958,24 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>63.78</v>
+        <v>64.03</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E90" t="n">
+        <v>79</v>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
@@ -3974,26 +3984,33 @@
         </is>
       </c>
       <c r="H90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>TOELY</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>06 AI Compute Silicon / Programmable logic</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>63.6</v>
+        <v>63.89</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E91" t="n">
+        <v>80</v>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
@@ -4007,16 +4024,16 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>UMAC</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>63.57</v>
+        <v>63.81</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -4024,7 +4041,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
@@ -4038,16 +4055,16 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>63.28</v>
+        <v>63.62</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -4055,7 +4072,7 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
@@ -4064,21 +4081,25 @@
         </is>
       </c>
       <c r="H93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>63</v>
+        <v>63.48</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -4086,7 +4107,7 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
@@ -4095,25 +4116,21 @@
         </is>
       </c>
       <c r="H94" t="inlineStr"/>
-      <c r="J94" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
-        </is>
-      </c>
+      <c r="J94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>62.87</v>
+        <v>63.21</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -4121,7 +4138,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
@@ -4135,16 +4152,16 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>RRC</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Financial software</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>62.83</v>
+        <v>63.01</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -4152,7 +4169,7 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
@@ -4166,21 +4183,24 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>6383.T</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>62.59</v>
+        <v>62.94</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E97" t="n">
+        <v>86</v>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
@@ -4194,16 +4214,16 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>62.47</v>
+        <v>62.83</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -4211,7 +4231,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
@@ -4225,16 +4245,16 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>SYM</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>62.38</v>
+        <v>62.8</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -4242,7 +4262,7 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
@@ -4256,24 +4276,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>6383.T</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>62.27</v>
+        <v>62.72</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E100" t="n">
-        <v>87</v>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
@@ -4287,16 +4304,16 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>62.25</v>
+        <v>62.69</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4304,7 +4321,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
@@ -4318,16 +4335,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>62.13</v>
+        <v>62.69</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4335,7 +4352,7 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
@@ -4349,21 +4366,24 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2252.HK</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>10 Models, Software &amp; Applications / Financial software</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>62.1</v>
+        <v>62.66</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E103" t="n">
+        <v>91</v>
       </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
@@ -4377,16 +4397,16 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>KTOS</t>
+          <t>SYM</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>62.06</v>
+        <v>62.5</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -4394,7 +4414,7 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
@@ -4417,7 +4437,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>61.98</v>
+        <v>62.49</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -4425,7 +4445,7 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
@@ -4439,7 +4459,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -4448,7 +4468,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>61.58</v>
+        <v>62.44</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4456,7 +4476,7 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
@@ -4470,16 +4490,16 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>61.52</v>
+        <v>62.33</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4487,7 +4507,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
@@ -4501,16 +4521,16 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>61.47</v>
+        <v>62.25</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -4518,7 +4538,7 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
@@ -4532,24 +4552,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>TOELY</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>61.42</v>
+        <v>61.92</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E109" t="n">
-        <v>95</v>
       </c>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
@@ -4563,16 +4580,16 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>KTOS</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>61.01</v>
+        <v>61.85</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -4580,7 +4597,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
@@ -4594,16 +4611,16 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>60.8</v>
+        <v>61.59</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -4611,7 +4628,7 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
@@ -4625,16 +4642,16 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>60.77</v>
+        <v>61.48</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -4642,7 +4659,7 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
@@ -4656,24 +4673,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>2252.HK</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>60.6</v>
+        <v>61.14</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E113" t="n">
-        <v>99</v>
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
@@ -4687,16 +4701,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>60.58</v>
+        <v>60.89</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4727,7 +4741,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>60.55</v>
+        <v>60.34</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -4749,24 +4763,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>6506.T</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>60.46</v>
+        <v>60.33</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E116" t="n">
-        <v>102</v>
       </c>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
@@ -4789,7 +4800,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>60.42</v>
+        <v>60.2</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -4808,16 +4819,16 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>PRCT</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>60.27</v>
+        <v>60.1</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -4825,7 +4836,7 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
@@ -4839,16 +4850,16 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>RRX</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>60.27</v>
+        <v>60.08</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -4856,7 +4867,7 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
@@ -4879,7 +4890,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>60.2</v>
+        <v>60.08</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -4887,7 +4898,7 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
@@ -4901,16 +4912,16 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>60.2</v>
+        <v>59.99</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -4918,7 +4929,7 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
@@ -4932,16 +4943,16 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>RRX</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>60.11</v>
+        <v>59.98</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -4949,7 +4960,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
@@ -4963,16 +4974,16 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>RRC</t>
+          <t>PRCT</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>59.69</v>
+        <v>59.95</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -4980,7 +4991,7 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
@@ -4994,16 +5005,16 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>AMKR</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>59.57</v>
+        <v>59.87</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -5011,7 +5022,7 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
@@ -5025,16 +5036,16 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>ALNT</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>59.39</v>
+        <v>59.79</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -5042,7 +5053,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
@@ -5056,21 +5067,24 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>6506.T</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>59.23</v>
+        <v>59.66</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E126" t="n">
+        <v>110</v>
       </c>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
@@ -5084,16 +5098,16 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>ASX</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI data layer</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>59.21</v>
+        <v>59.56</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -5115,16 +5129,16 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>UCTT</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>59.1</v>
+        <v>59.17</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -5146,16 +5160,16 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>CARR</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>59</v>
+        <v>59.03</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
@@ -5177,16 +5191,16 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ALNT</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>58.88</v>
+        <v>58.95</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -5208,16 +5222,16 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI commerce</t>
+          <t>10 Models, Software &amp; Applications / AI data layer</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>58.84</v>
+        <v>58.79</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -5239,21 +5253,24 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>KGX.DE</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>58.72</v>
+        <v>58.75</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E132" t="n">
+        <v>116</v>
       </c>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
@@ -5284,7 +5301,7 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
@@ -5298,21 +5315,24 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>6481.T</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>10 Models, Software &amp; Applications / AI commerce</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>58.5</v>
+        <v>58.61</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E134" t="n">
+        <v>118</v>
       </c>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
@@ -5326,16 +5346,16 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>58.4</v>
+        <v>58.52</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -5343,7 +5363,7 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
@@ -5357,16 +5377,16 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>58.33</v>
+        <v>58.5</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
@@ -5374,7 +5394,7 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
@@ -5388,16 +5408,16 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>WYFI</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>58.11</v>
+        <v>58.5</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
@@ -5405,7 +5425,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
@@ -5419,7 +5439,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -5428,7 +5448,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>58.01</v>
+        <v>58.43</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
@@ -5436,7 +5456,7 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
@@ -5450,16 +5470,16 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>57.89</v>
+        <v>58.37</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
@@ -5467,7 +5487,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
@@ -5481,16 +5501,16 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>AMKR</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>57.82</v>
+        <v>57.86</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
@@ -5498,7 +5518,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
@@ -5512,16 +5532,16 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>57.81</v>
+        <v>57.83</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -5529,7 +5549,7 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
@@ -5543,16 +5563,16 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>WYFI</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>57.67</v>
+        <v>57.77</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
@@ -5560,7 +5580,7 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
@@ -5574,16 +5594,16 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ASX</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>57.61</v>
+        <v>57.75</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -5591,7 +5611,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
@@ -5605,16 +5625,16 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>57.57</v>
+        <v>57.74</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
@@ -5622,7 +5642,7 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
@@ -5645,7 +5665,7 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>57.49</v>
+        <v>57.73</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
@@ -5664,16 +5684,16 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ONDS</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>57.45</v>
+        <v>57.64</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
@@ -5681,7 +5701,7 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
@@ -5695,16 +5715,16 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>ONDS</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Consumer fintech (AI adopter)</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>57.15</v>
+        <v>57.38</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
@@ -5712,7 +5732,7 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
@@ -5726,16 +5746,16 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>57.12</v>
+        <v>57.33</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
@@ -5743,7 +5763,7 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr">
@@ -5757,16 +5777,16 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>57.11</v>
+        <v>57.07</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
@@ -5774,7 +5794,7 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr">
@@ -5788,12 +5808,12 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>AVAV</t>
+          <t>PSIX</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -5805,7 +5825,7 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
@@ -5819,24 +5839,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>CARR</t>
+          <t>6481.T</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>56.71</v>
+        <v>56.76</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E151" t="n">
-        <v>132</v>
       </c>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
@@ -5850,16 +5867,16 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>HIVE</t>
+          <t>PPL</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>56.62</v>
+        <v>56.74</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -5867,7 +5884,7 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
@@ -5881,16 +5898,16 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>PPL</t>
+          <t>AVAV</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>56.52</v>
+        <v>56.67</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -5898,7 +5915,7 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
@@ -5912,16 +5929,16 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>TKR</t>
+          <t>HIVE</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>56.48</v>
+        <v>56.62</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -5929,7 +5946,7 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
@@ -5943,16 +5960,16 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>TNC</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Humanoid &amp; service robot makers</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>56.21</v>
+        <v>56.56</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
@@ -5960,7 +5977,7 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
@@ -5974,16 +5991,16 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>PSIX</t>
+          <t>TKR</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>55.93</v>
+        <v>56.55</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
@@ -5991,7 +6008,7 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
@@ -6005,16 +6022,16 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>55.71</v>
+        <v>56.55</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
@@ -6022,7 +6039,7 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
@@ -6036,21 +6053,24 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>6324.T</t>
+          <t>TNC</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>11 Robotics &amp; Physical AI / Humanoid &amp; service robot makers</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>55.69</v>
+        <v>56.09</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E158" t="n">
+        <v>140</v>
       </c>
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
@@ -6064,16 +6084,16 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>UCTT</t>
+          <t>VPG</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>55.69</v>
+        <v>56.04</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
@@ -6081,7 +6101,7 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
@@ -6095,16 +6115,16 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>55.45</v>
+        <v>56</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
@@ -6112,7 +6132,7 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
@@ -6126,16 +6146,16 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2590.HK</t>
+          <t>MELE.BR</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>06 AI Compute Silicon / Magnetic &amp; position sensing (robotics)</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>55.27</v>
+        <v>55.83</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
@@ -6154,24 +6174,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>BW</t>
+          <t>2590.HK</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>55.17</v>
+        <v>55.51</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E162" t="n">
-        <v>141</v>
       </c>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
@@ -6185,16 +6202,16 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>BW</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>55.14</v>
+        <v>55.51</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
@@ -6202,7 +6219,7 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
@@ -6212,6 +6229,96 @@
       </c>
       <c r="H163" t="inlineStr"/>
       <c r="J163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>55.44</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>144</v>
+      </c>
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr"/>
+      <c r="J164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>CAMT</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>55.26</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>145</v>
+      </c>
+      <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr"/>
+      <c r="J165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>6324.T</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr"/>
+      <c r="J166" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
rescore 2026-10-30: refresh prices and scores for all names (#230)
Full objective, 50DMA and reverse-DCF refresh after 179 names had gone
stale since 2026-10-11. Model adds VRT and ASML; MU moves to the top
tier; WDC and LRCX exit clocks start.

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-29 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-10-30 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J163"/>
+  <dimension ref="A1:J166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1068,7 +1068,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-10-29, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-10-30, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1127,16 +1127,16 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>06 Silicon - Memory</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>85.53</v>
+        <v>88.7</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1158,31 +1158,27 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
-        </is>
-      </c>
+        <v>5.26</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>83.87</v>
+        <v>85.27</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓✓✓</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1200,23 +1196,27 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J4" t="inlineStr"/>
+        <v>5.26</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>82.38</v>
+        <v>83.64</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1238,23 +1238,23 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>81.90000000000001</v>
+        <v>82.95999999999999</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1276,27 +1276,23 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
-        </is>
-      </c>
+        <v>5.26</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>81.58</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1318,27 +1314,27 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
+          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>79.79000000000001</v>
+        <v>82.20999999999999</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1360,9 +1356,13 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J8" t="inlineStr"/>
+        <v>5.26</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>79.79000000000001</v>
+        <v>80.79000000000001</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1398,23 +1398,23 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>79.53</v>
+        <v>80.43000000000001</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1436,23 +1436,23 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>79.15000000000001</v>
+        <v>79.12</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1474,23 +1474,23 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06 Silicon - Memory</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>78.39</v>
+        <v>78.73</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1512,23 +1512,23 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>RDDT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>76.27</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1550,23 +1550,23 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>75.8</v>
+        <v>76.02</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1588,23 +1588,27 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J14" t="inlineStr"/>
+        <v>5.26</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RDDT</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>75.53</v>
+        <v>75.79000000000001</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1626,23 +1630,23 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>74.79000000000001</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1664,23 +1668,23 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>5.88</v>
+        <v>5.26</v>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>74.48</v>
+        <v>74.73999999999999</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1692,7 +1696,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ENTER (rank 15, score 74.5)</t>
+          <t>ENTER (rank 15, score 74.7)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1702,55 +1706,61 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+        <v>5.26</v>
+      </c>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>6861.T</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>03 DC Infrastructure</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>74.28</v>
+        <v>74.5</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="E18" t="n">
+        <v>16</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
+      <c r="I18" t="n">
+        <v>5.26</v>
+      </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>74.03</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1758,75 +1768,58 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>16</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="n">
-        <v>5.88</v>
-      </c>
       <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GMED</t>
+          <t>6861.T</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>73.92</v>
+        <v>73.73</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E20" t="n">
-        <v>17</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="n">
-        <v>5.88</v>
-      </c>
       <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>GMED</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>73.75</v>
+        <v>73.42</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1836,33 +1829,43 @@
       <c r="E21" t="n">
         <v>18</v>
       </c>
-      <c r="F21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
+      <c r="I21" t="n">
+        <v>5.26</v>
+      </c>
       <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>73.51000000000001</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
+      </c>
+      <c r="E22" t="n">
+        <v>19</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
@@ -1876,16 +1879,16 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>73.40000000000001</v>
+        <v>73.16</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1893,7 +1896,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
@@ -1907,16 +1910,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>72.98999999999999</v>
+        <v>72.89</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1924,26 +1927,33 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>20</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>EXIT PENDING (rank 21 &gt; exit rank 18, since 2026-10-30)</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
+      <c r="I24" t="n">
+        <v>5.26</v>
+      </c>
       <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>03 DC Infrastructure</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1955,7 +1965,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
@@ -1969,16 +1979,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>72.64</v>
+        <v>72.70999999999999</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1986,7 +1996,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
@@ -2000,24 +2010,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>72.38</v>
+        <v>72.66</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
-      </c>
-      <c r="E27" t="n">
-        <v>23</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
@@ -2031,16 +2038,16 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>72.25</v>
+        <v>72.28</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2050,28 +2057,35 @@
       <c r="E28" t="n">
         <v>24</v>
       </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>EXIT PENDING (rank 24 &gt; exit rank 18, since 2026-10-30)</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
+      <c r="I28" t="n">
+        <v>5.26</v>
+      </c>
       <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>71.88</v>
+        <v>72.08</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2102,7 +2116,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>71.58</v>
+        <v>72.08</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2124,16 +2138,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>71.45</v>
+        <v>71.48</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2155,16 +2169,16 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>71.09999999999999</v>
+        <v>71.17</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2186,21 +2200,24 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BSL.DE</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>70.95999999999999</v>
+        <v>70.64</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
+      </c>
+      <c r="E33" t="n">
+        <v>29</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
@@ -2214,24 +2231,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>6954.T</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>70.68000000000001</v>
+        <v>70.63</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
-      </c>
-      <c r="E34" t="n">
-        <v>29</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
@@ -2245,7 +2259,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2254,11 +2268,11 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>69.26000000000001</v>
+        <v>70.55</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -2276,20 +2290,20 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>HTHIY</t>
+          <t>BSL.DE</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>69.17</v>
+        <v>70.36</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -2304,7 +2318,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2313,11 +2327,11 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>69.17</v>
+        <v>70.11</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -2335,16 +2349,16 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>69.15000000000001</v>
+        <v>69.91</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2366,16 +2380,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CGNX</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>68.88</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2397,16 +2411,16 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>68.86</v>
+        <v>69.69</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2428,16 +2442,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>68.45999999999999</v>
+        <v>69.45</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2459,16 +2473,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>68.45999999999999</v>
+        <v>69.44</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2490,24 +2504,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>HTHIY</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>68.31999999999999</v>
+        <v>69.33</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E43" t="n">
-        <v>37</v>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
@@ -2516,25 +2527,21 @@
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
-        </is>
-      </c>
+      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>CGNX</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>68.31</v>
+        <v>69.15000000000001</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2542,7 +2549,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
@@ -2556,16 +2563,16 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>NOVT</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>68.20999999999999</v>
+        <v>69.11</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2573,7 +2580,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
@@ -2587,16 +2594,16 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>68</v>
+        <v>68.77</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2604,7 +2611,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
@@ -2618,16 +2625,16 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>6268.T</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>67.98</v>
+        <v>68.73</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2646,16 +2653,16 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>67.95</v>
+        <v>68.43000000000001</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2663,7 +2670,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
@@ -2677,16 +2684,16 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>NTAP</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>67.73</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2694,7 +2701,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
@@ -2708,16 +2715,16 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>67.7</v>
+        <v>67.98999999999999</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2725,7 +2732,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
@@ -2739,16 +2746,16 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>67.42</v>
+        <v>67.81999999999999</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2756,7 +2763,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
@@ -2765,25 +2772,21 @@
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
-        </is>
-      </c>
+      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>67.22</v>
+        <v>67.73999999999999</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -2791,7 +2794,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
@@ -2805,16 +2808,16 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>NOVT</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>67.15000000000001</v>
+        <v>67.69</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -2822,7 +2825,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
@@ -2836,16 +2839,16 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MKSI</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>67</v>
+        <v>67.56999999999999</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2853,7 +2856,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
@@ -2867,16 +2870,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>WDAY</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
+          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>67</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2884,7 +2887,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
@@ -2898,21 +2901,24 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>6954.T</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>66.83</v>
+        <v>67.51000000000001</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E56" t="n">
+        <v>48</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
@@ -2921,21 +2927,25 @@
         </is>
       </c>
       <c r="H56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>66.73</v>
+        <v>67.34</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -2952,21 +2962,25 @@
         </is>
       </c>
       <c r="H57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>10 Models, Software &amp; Applications / Consumer fintech (AI adopter)</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>66.72</v>
+        <v>67.23999999999999</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2988,16 +3002,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>66.65000000000001</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3019,16 +3033,16 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>66.27</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3050,16 +3064,16 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>66.20999999999999</v>
+        <v>67.14</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -3081,16 +3095,16 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>AUTO.OL</t>
+          <t>6268.T</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>66.13</v>
+        <v>66.97</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3109,16 +3123,16 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>66.02</v>
+        <v>66.77</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3140,16 +3154,16 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>65.95999999999999</v>
+        <v>66.66</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3171,16 +3185,16 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>MKSI</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>65.67</v>
+        <v>66.36</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3202,16 +3216,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>65.61</v>
+        <v>66.31999999999999</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3233,16 +3247,16 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>65.31</v>
+        <v>66.3</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3264,24 +3278,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>OUST</t>
+          <t>AUTO.OL</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>65.20999999999999</v>
+        <v>66.27</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E68" t="n">
-        <v>59</v>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
@@ -3295,16 +3306,16 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>65.04000000000001</v>
+        <v>66.2</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3312,7 +3323,7 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
@@ -3326,16 +3337,16 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>65.02</v>
+        <v>65.95999999999999</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3343,7 +3354,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
@@ -3357,16 +3368,16 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>64.88</v>
+        <v>65.95</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3374,7 +3385,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
@@ -3388,16 +3399,16 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>64.75</v>
+        <v>65.79000000000001</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3405,7 +3416,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
@@ -3419,16 +3430,16 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>64.73999999999999</v>
+        <v>65.73</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3436,7 +3447,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
@@ -3450,21 +3461,24 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>64.69</v>
+        <v>65.45</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E74" t="n">
+        <v>64</v>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
@@ -3478,16 +3492,16 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>64.56999999999999</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3509,16 +3523,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>64.56</v>
+        <v>65.27</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3540,16 +3554,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>64.52</v>
+        <v>65.26000000000001</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3571,16 +3585,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>64.47</v>
+        <v>65.06999999999999</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3597,25 +3611,21 @@
         </is>
       </c>
       <c r="H78" t="inlineStr"/>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
+      <c r="J78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>64.44</v>
+        <v>65.04000000000001</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3637,16 +3647,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>64.43000000000001</v>
+        <v>65.02</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3668,16 +3678,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>OUST</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>64.38</v>
+        <v>64.97</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3699,16 +3709,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>64.36</v>
+        <v>64.88</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3730,24 +3740,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>64.34</v>
+        <v>64.5</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E83" t="n">
-        <v>73</v>
       </c>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
@@ -3761,16 +3768,16 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>GNRC</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>64.28</v>
+        <v>64.37</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -3778,7 +3785,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
@@ -3792,16 +3799,16 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>64.15000000000001</v>
+        <v>64.34999999999999</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -3809,7 +3816,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
@@ -3818,25 +3825,21 @@
         </is>
       </c>
       <c r="H85" t="inlineStr"/>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
-        </is>
-      </c>
+      <c r="J85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>PLAB</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>64.08</v>
+        <v>64.33</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3844,7 +3847,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
@@ -3858,16 +3861,16 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Programmable logic</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>63.92</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3875,7 +3878,7 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
@@ -3889,16 +3892,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>UMAC</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>63.86</v>
+        <v>64.27</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3906,7 +3909,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
@@ -3915,21 +3918,25 @@
         </is>
       </c>
       <c r="H88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>PLAB</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>63.84</v>
+        <v>64.17</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3937,7 +3944,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
@@ -3951,21 +3958,24 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>63.78</v>
+        <v>64.03</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E90" t="n">
+        <v>79</v>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
@@ -3974,26 +3984,33 @@
         </is>
       </c>
       <c r="H90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>TOELY</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>06 AI Compute Silicon / Programmable logic</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>63.6</v>
+        <v>63.89</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E91" t="n">
+        <v>80</v>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
@@ -4007,16 +4024,16 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>UMAC</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>63.57</v>
+        <v>63.81</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -4024,7 +4041,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
@@ -4038,16 +4055,16 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>63.28</v>
+        <v>63.62</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -4055,7 +4072,7 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
@@ -4064,21 +4081,25 @@
         </is>
       </c>
       <c r="H93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>63</v>
+        <v>63.48</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -4086,7 +4107,7 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
@@ -4095,25 +4116,21 @@
         </is>
       </c>
       <c r="H94" t="inlineStr"/>
-      <c r="J94" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
-        </is>
-      </c>
+      <c r="J94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>62.87</v>
+        <v>63.21</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -4121,7 +4138,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
@@ -4135,16 +4152,16 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>RRC</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Financial software</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>62.83</v>
+        <v>63.01</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -4152,7 +4169,7 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
@@ -4166,21 +4183,24 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>6383.T</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>62.59</v>
+        <v>62.94</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E97" t="n">
+        <v>86</v>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
@@ -4194,16 +4214,16 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>62.47</v>
+        <v>62.83</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -4211,7 +4231,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
@@ -4225,16 +4245,16 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>SYM</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>62.38</v>
+        <v>62.8</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -4242,7 +4262,7 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
@@ -4256,24 +4276,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>6383.T</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>62.27</v>
+        <v>62.72</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E100" t="n">
-        <v>87</v>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
@@ -4287,16 +4304,16 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>62.25</v>
+        <v>62.69</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4304,7 +4321,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
@@ -4318,16 +4335,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>62.13</v>
+        <v>62.69</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4335,7 +4352,7 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
@@ -4349,21 +4366,24 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2252.HK</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>10 Models, Software &amp; Applications / Financial software</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>62.1</v>
+        <v>62.66</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E103" t="n">
+        <v>91</v>
       </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
@@ -4377,16 +4397,16 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>KTOS</t>
+          <t>SYM</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>62.06</v>
+        <v>62.5</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -4394,7 +4414,7 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
@@ -4417,7 +4437,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>61.98</v>
+        <v>62.49</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -4425,7 +4445,7 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
@@ -4439,7 +4459,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -4448,7 +4468,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>61.58</v>
+        <v>62.44</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4456,7 +4476,7 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
@@ -4470,16 +4490,16 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>61.52</v>
+        <v>62.33</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4487,7 +4507,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
@@ -4501,16 +4521,16 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>61.47</v>
+        <v>62.25</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -4518,7 +4538,7 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
@@ -4532,24 +4552,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>TOELY</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>61.42</v>
+        <v>61.92</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E109" t="n">
-        <v>95</v>
       </c>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
@@ -4563,16 +4580,16 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>KTOS</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>61.01</v>
+        <v>61.85</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -4580,7 +4597,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
@@ -4594,16 +4611,16 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>60.8</v>
+        <v>61.59</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -4611,7 +4628,7 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
@@ -4625,16 +4642,16 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>60.77</v>
+        <v>61.48</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -4642,7 +4659,7 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
@@ -4656,24 +4673,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>2252.HK</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>60.6</v>
+        <v>61.14</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E113" t="n">
-        <v>99</v>
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
@@ -4687,16 +4701,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>60.58</v>
+        <v>60.89</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4727,7 +4741,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>60.55</v>
+        <v>60.34</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -4749,24 +4763,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>6506.T</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>60.46</v>
+        <v>60.33</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E116" t="n">
-        <v>102</v>
       </c>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
@@ -4789,7 +4800,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>60.42</v>
+        <v>60.2</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -4808,16 +4819,16 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>PRCT</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>60.27</v>
+        <v>60.1</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -4825,7 +4836,7 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
@@ -4839,16 +4850,16 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>RRX</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>60.27</v>
+        <v>60.08</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -4856,7 +4867,7 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
@@ -4879,7 +4890,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>60.2</v>
+        <v>60.08</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -4887,7 +4898,7 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
@@ -4901,16 +4912,16 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>60.2</v>
+        <v>59.99</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -4918,7 +4929,7 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
@@ -4932,16 +4943,16 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>RRX</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>60.11</v>
+        <v>59.98</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -4949,7 +4960,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
@@ -4963,16 +4974,16 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>RRC</t>
+          <t>PRCT</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>59.69</v>
+        <v>59.95</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -4980,7 +4991,7 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
@@ -4994,16 +5005,16 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>AMKR</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>59.57</v>
+        <v>59.87</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -5011,7 +5022,7 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
@@ -5025,16 +5036,16 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>ALNT</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>59.39</v>
+        <v>59.79</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -5042,7 +5053,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
@@ -5056,21 +5067,24 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>6506.T</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>59.23</v>
+        <v>59.66</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E126" t="n">
+        <v>110</v>
       </c>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
@@ -5084,16 +5098,16 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>ASX</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI data layer</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>59.21</v>
+        <v>59.56</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -5115,16 +5129,16 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>UCTT</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>59.1</v>
+        <v>59.17</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -5146,16 +5160,16 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>CARR</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>59</v>
+        <v>59.03</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
@@ -5177,16 +5191,16 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ALNT</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>58.88</v>
+        <v>58.95</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -5208,16 +5222,16 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI commerce</t>
+          <t>10 Models, Software &amp; Applications / AI data layer</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>58.84</v>
+        <v>58.79</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -5239,21 +5253,24 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>KGX.DE</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>58.72</v>
+        <v>58.75</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E132" t="n">
+        <v>116</v>
       </c>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
@@ -5284,7 +5301,7 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
@@ -5298,21 +5315,24 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>6481.T</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>10 Models, Software &amp; Applications / AI commerce</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>58.5</v>
+        <v>58.61</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E134" t="n">
+        <v>118</v>
       </c>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
@@ -5326,16 +5346,16 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>58.4</v>
+        <v>58.52</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -5343,7 +5363,7 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
@@ -5357,16 +5377,16 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>58.33</v>
+        <v>58.5</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
@@ -5374,7 +5394,7 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
@@ -5388,16 +5408,16 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>WYFI</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>58.11</v>
+        <v>58.5</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
@@ -5405,7 +5425,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
@@ -5419,7 +5439,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -5428,7 +5448,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>58.01</v>
+        <v>58.43</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
@@ -5436,7 +5456,7 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
@@ -5450,16 +5470,16 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>57.89</v>
+        <v>58.37</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
@@ -5467,7 +5487,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
@@ -5481,16 +5501,16 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>AMKR</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>57.82</v>
+        <v>57.86</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
@@ -5498,7 +5518,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
@@ -5512,16 +5532,16 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>57.81</v>
+        <v>57.83</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -5529,7 +5549,7 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
@@ -5543,16 +5563,16 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>WYFI</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>57.67</v>
+        <v>57.77</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
@@ -5560,7 +5580,7 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
@@ -5574,16 +5594,16 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ASX</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>57.61</v>
+        <v>57.75</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -5591,7 +5611,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
@@ -5605,16 +5625,16 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>57.57</v>
+        <v>57.74</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
@@ -5622,7 +5642,7 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
@@ -5645,7 +5665,7 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>57.49</v>
+        <v>57.73</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
@@ -5664,16 +5684,16 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ONDS</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>57.45</v>
+        <v>57.64</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
@@ -5681,7 +5701,7 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
@@ -5695,16 +5715,16 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>ONDS</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Consumer fintech (AI adopter)</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>57.15</v>
+        <v>57.38</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
@@ -5712,7 +5732,7 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
@@ -5726,16 +5746,16 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>57.12</v>
+        <v>57.33</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
@@ -5743,7 +5763,7 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr">
@@ -5757,16 +5777,16 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>57.11</v>
+        <v>57.07</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
@@ -5774,7 +5794,7 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr">
@@ -5788,12 +5808,12 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>AVAV</t>
+          <t>PSIX</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -5805,7 +5825,7 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
@@ -5819,24 +5839,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>CARR</t>
+          <t>6481.T</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>56.71</v>
+        <v>56.76</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E151" t="n">
-        <v>132</v>
       </c>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
@@ -5850,16 +5867,16 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>HIVE</t>
+          <t>PPL</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>56.62</v>
+        <v>56.74</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -5867,7 +5884,7 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
@@ -5881,16 +5898,16 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>PPL</t>
+          <t>AVAV</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>56.52</v>
+        <v>56.67</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -5898,7 +5915,7 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
@@ -5912,16 +5929,16 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>TKR</t>
+          <t>HIVE</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>56.48</v>
+        <v>56.62</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -5929,7 +5946,7 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
@@ -5943,16 +5960,16 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>TNC</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Humanoid &amp; service robot makers</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>56.21</v>
+        <v>56.56</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
@@ -5960,7 +5977,7 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
@@ -5974,16 +5991,16 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>PSIX</t>
+          <t>TKR</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>55.93</v>
+        <v>56.55</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
@@ -5991,7 +6008,7 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
@@ -6005,16 +6022,16 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>55.71</v>
+        <v>56.55</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
@@ -6022,7 +6039,7 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
@@ -6036,21 +6053,24 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>6324.T</t>
+          <t>TNC</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>11 Robotics &amp; Physical AI / Humanoid &amp; service robot makers</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>55.69</v>
+        <v>56.09</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E158" t="n">
+        <v>140</v>
       </c>
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
@@ -6064,16 +6084,16 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>UCTT</t>
+          <t>VPG</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>55.69</v>
+        <v>56.04</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
@@ -6081,7 +6101,7 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
@@ -6095,16 +6115,16 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>55.45</v>
+        <v>56</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
@@ -6112,7 +6132,7 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
@@ -6126,16 +6146,16 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2590.HK</t>
+          <t>MELE.BR</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>06 AI Compute Silicon / Magnetic &amp; position sensing (robotics)</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>55.27</v>
+        <v>55.83</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
@@ -6154,24 +6174,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>BW</t>
+          <t>2590.HK</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>55.17</v>
+        <v>55.51</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E162" t="n">
-        <v>141</v>
       </c>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
@@ -6185,16 +6202,16 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>BW</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>55.14</v>
+        <v>55.51</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
@@ -6202,7 +6219,7 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
@@ -6212,6 +6229,96 @@
       </c>
       <c r="H163" t="inlineStr"/>
       <c r="J163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>55.44</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>144</v>
+      </c>
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr"/>
+      <c r="J164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>CAMT</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>55.26</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>145</v>
+      </c>
+      <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr"/>
+      <c r="J165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>6324.T</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr"/>
+      <c r="J166" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
weekly-scan 2026-10-31: 48 earnings refreshes, RDDT+LRCX exit (ticket HELD), EQT-RRC merger
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-30 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-10-31 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J166"/>
+  <dimension ref="A1:J167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1068,7 +1068,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-10-30, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-10-31, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>88.7</v>
+        <v>88.62</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -1207,16 +1207,16 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>83.64</v>
+        <v>83.79000000000001</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1238,23 +1238,27 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>5.26</v>
-      </c>
-      <c r="J5" t="inlineStr"/>
+        <v>5.88</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>82.95999999999999</v>
+        <v>83.34</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1276,23 +1280,23 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>82.34999999999999</v>
+        <v>82.95999999999999</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1314,13 +1318,9 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>5.26</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
-        </is>
-      </c>
+        <v>5.88</v>
+      </c>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -1367,16 +1367,16 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>80.79000000000001</v>
+        <v>80.43000000000001</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1398,23 +1398,23 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>80.43000000000001</v>
+        <v>80.29000000000001</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1436,23 +1436,23 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>79.12</v>
+        <v>78.58</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1474,23 +1474,23 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>78.73</v>
+        <v>76.02</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1512,23 +1512,27 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.26</v>
-      </c>
-      <c r="J12" t="inlineStr"/>
+        <v>5.88</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RDDT</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>77.09999999999999</v>
+        <v>75.79000000000001</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1550,23 +1554,23 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>76.02</v>
+        <v>74.94</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1588,27 +1592,23 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.26</v>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+        <v>5.88</v>
+      </c>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>75.79000000000001</v>
+        <v>74.63</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1630,23 +1630,23 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>74.84999999999999</v>
+        <v>74.62</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1668,23 +1668,23 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 DC Infrastructure</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>74.73999999999999</v>
+        <v>74.5</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ENTER (rank 15, score 74.7)</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1706,23 +1706,23 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>03 DC Infrastructure</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>74.5</v>
+        <v>74.20999999999999</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1732,20 +1732,13 @@
       <c r="E18" t="n">
         <v>16</v>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="n">
-        <v>5.26</v>
-      </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1810,16 +1803,16 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GMED</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>73.42</v>
+        <v>73.54000000000001</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1841,23 +1834,23 @@
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>GMED</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>73.34999999999999</v>
+        <v>73.42</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1867,28 +1860,35 @@
       <c r="E22" t="n">
         <v>19</v>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>EXIT PENDING (rank 19 &gt; exit rank 18, since 2026-10-31)</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
+      <c r="I22" t="n">
+        <v>5.88</v>
+      </c>
       <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>73.16</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1910,16 +1910,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>RDDT</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>72.89</v>
+        <v>73.3</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1931,18 +1931,15 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>EXIT PENDING (rank 21 &gt; exit rank 18, since 2026-10-30)</t>
+          <t>EXIT (pending since 2026-10-30, confirmed)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="I24" t="n">
-        <v>5.26</v>
-      </c>
       <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1979,24 +1976,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>72.70999999999999</v>
+        <v>72.66</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
-      </c>
-      <c r="E26" t="n">
-        <v>23</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
@@ -2010,21 +2004,24 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>72.66</v>
+        <v>72.64</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
+      </c>
+      <c r="E27" t="n">
+        <v>23</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
@@ -2059,18 +2056,15 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>EXIT PENDING (rank 24 &gt; exit rank 18, since 2026-10-30)</t>
+          <t>EXIT (pending since 2026-10-30, confirmed)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" t="n">
-        <v>5.26</v>
-      </c>
       <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
@@ -2209,7 +2203,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>70.64</v>
+        <v>71.14</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2231,21 +2225,24 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>6954.T</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>70.63</v>
+        <v>71.09</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
+      </c>
+      <c r="E34" t="n">
+        <v>30</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
@@ -2259,24 +2256,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>6954.T</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>70.55</v>
+        <v>70.63</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
-      </c>
-      <c r="E35" t="n">
-        <v>30</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
@@ -2318,16 +2312,16 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>70.11</v>
+        <v>70.25</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2349,20 +2343,20 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>69.91</v>
+        <v>70.11</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -2380,16 +2374,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>69.70999999999999</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2411,16 +2405,16 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>69.69</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2442,16 +2436,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>69.45</v>
+        <v>69.69</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2473,16 +2467,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>69.44</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2594,24 +2588,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>68.77</v>
+        <v>68.55</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E46" t="n">
-        <v>39</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
@@ -2625,21 +2616,24 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>68.73</v>
+        <v>68.43000000000001</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E47" t="n">
+        <v>39</v>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
@@ -2653,16 +2647,16 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>68.43000000000001</v>
+        <v>68.41</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2777,16 +2771,16 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>NOVT</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>67.73999999999999</v>
+        <v>67.69</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -2808,16 +2802,16 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>NOVT</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>67.69</v>
+        <v>67.62</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -2839,16 +2833,16 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>67.56999999999999</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2870,16 +2864,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>67.54000000000001</v>
+        <v>67.56999999999999</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2971,16 +2965,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Consumer fintech (AI adopter)</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>67.23999999999999</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -3002,16 +2996,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>67.18000000000001</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3033,16 +3027,16 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>67.15000000000001</v>
+        <v>67.14</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3064,24 +3058,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>6268.T</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>67.14</v>
+        <v>66.97</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E61" t="n">
-        <v>53</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
@@ -3095,21 +3086,24 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>6268.T</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>66.97</v>
+        <v>66.77</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E62" t="n">
+        <v>53</v>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
@@ -3123,16 +3117,16 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / Consumer fintech (AI adopter)</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>66.77</v>
+        <v>66.73999999999999</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3315,7 +3309,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>66.2</v>
+        <v>66.03</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3377,7 +3371,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>65.95</v>
+        <v>65.81</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3439,7 +3433,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>65.73</v>
+        <v>65.5</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3470,7 +3464,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>65.45</v>
+        <v>65.48999999999999</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -3492,16 +3486,16 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>65.29000000000001</v>
+        <v>65.27</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3523,16 +3517,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>65.27</v>
+        <v>65.23</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3554,16 +3548,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>GNRC</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>65.26000000000001</v>
+        <v>65.04000000000001</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3585,16 +3579,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>65.06999999999999</v>
+        <v>65.02</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3616,16 +3610,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>OUST</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>65.04000000000001</v>
+        <v>64.97</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3647,16 +3641,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>65.02</v>
+        <v>64.95</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3678,16 +3672,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>OUST</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>64.97</v>
+        <v>64.88</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3709,16 +3703,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>64.88</v>
+        <v>64.53</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3740,21 +3734,24 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>64.5</v>
+        <v>64.48</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E83" t="n">
+        <v>73</v>
       </c>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
@@ -3785,7 +3782,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
@@ -3816,7 +3813,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
@@ -3830,16 +3827,16 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>64.33</v>
+        <v>64.27</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3847,7 +3844,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
@@ -3856,21 +3853,25 @@
         </is>
       </c>
       <c r="H86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>64.29000000000001</v>
+        <v>64.27</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3878,7 +3879,7 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
@@ -3892,16 +3893,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>PLAB</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>64.27</v>
+        <v>64.17</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3909,7 +3910,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
@@ -3918,33 +3919,26 @@
         </is>
       </c>
       <c r="H88" t="inlineStr"/>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
+      <c r="J88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>PLAB</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>64.17</v>
+        <v>64.14</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E89" t="n">
-        <v>78</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
@@ -3967,7 +3961,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>64.03</v>
+        <v>64.06</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -4099,7 +4093,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>63.48</v>
+        <v>63.51</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -4161,7 +4155,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>63.01</v>
+        <v>63.05</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -4304,12 +4298,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -4335,16 +4329,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>10 Models, Software &amp; Applications / Financial software</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>62.69</v>
+        <v>62.66</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4366,12 +4360,12 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Financial software</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -4459,16 +4453,16 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>62.44</v>
+        <v>62.33</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4490,16 +4484,16 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>62.33</v>
+        <v>62.23</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4521,16 +4515,16 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>62.25</v>
+        <v>62.06</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -4611,16 +4605,16 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>61.59</v>
+        <v>61.47</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -4642,24 +4636,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>2252.HK</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>61.48</v>
+        <v>61.14</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E112" t="n">
-        <v>99</v>
       </c>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
@@ -4673,21 +4664,24 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2252.HK</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>61.14</v>
+        <v>61.09</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E113" t="n">
+        <v>99</v>
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
@@ -4701,16 +4695,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>60.89</v>
+        <v>60.47</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4881,16 +4875,16 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>MBLY</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>60.08</v>
+        <v>59.98</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -4912,16 +4906,16 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>PRCT</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>59.99</v>
+        <v>59.95</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -4943,16 +4937,16 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>59.98</v>
+        <v>59.89</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -4974,16 +4968,16 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>PRCT</t>
+          <t>ALNT</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>59.95</v>
+        <v>59.87</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -5005,16 +4999,16 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>MBLY</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>59.87</v>
+        <v>59.86</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -5036,16 +5030,16 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>ALNT</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>59.79</v>
+        <v>59.66</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -5067,16 +5061,16 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>ASX</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>59.66</v>
+        <v>59.56</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -5098,16 +5092,16 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ASX</t>
+          <t>UCTT</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>59.56</v>
+        <v>59.17</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -5129,16 +5123,16 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>UCTT</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>59.17</v>
+        <v>59.11</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -5200,7 +5194,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>58.95</v>
+        <v>58.93</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -5346,16 +5340,16 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>58.52</v>
+        <v>58.56</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -5448,7 +5442,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>58.43</v>
+        <v>58.5</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
@@ -5470,16 +5464,16 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>AMKR</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>58.37</v>
+        <v>57.86</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
@@ -5501,16 +5495,16 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>AMKR</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>57.86</v>
+        <v>57.8</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
@@ -5532,7 +5526,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -5541,7 +5535,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>57.83</v>
+        <v>57.75</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -5563,24 +5557,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>DRO.AX</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>57.77</v>
+        <v>57.73</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E142" t="n">
-        <v>126</v>
       </c>
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
@@ -5594,7 +5585,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -5603,7 +5594,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>57.75</v>
+        <v>57.65</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -5611,7 +5602,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
@@ -5625,16 +5616,16 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>57.74</v>
+        <v>57.64</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
@@ -5642,7 +5633,7 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
@@ -5656,7 +5647,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>DRO.AX</t>
+          <t>ONDS</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -5665,12 +5656,15 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>57.73</v>
+        <v>57.53</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E145" t="n">
+        <v>128</v>
       </c>
       <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
@@ -5684,16 +5678,16 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>57.64</v>
+        <v>57.33</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
@@ -5715,16 +5709,16 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>ONDS</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>57.38</v>
+        <v>57.02</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
@@ -5746,16 +5740,16 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>PSIX</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>57.33</v>
+        <v>56.87</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
@@ -5777,16 +5771,16 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>PPL</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>57.07</v>
+        <v>56.8</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
@@ -5808,24 +5802,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>PSIX</t>
+          <t>6481.T</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>56.81</v>
+        <v>56.76</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E150" t="n">
-        <v>133</v>
       </c>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
@@ -5839,21 +5830,24 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>6481.T</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>56.76</v>
+        <v>56.67</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E151" t="n">
+        <v>133</v>
       </c>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
@@ -5867,16 +5861,16 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>PPL</t>
+          <t>AVAV</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>56.74</v>
+        <v>56.67</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -5898,16 +5892,16 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>AVAV</t>
+          <t>HIVE</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>56.67</v>
+        <v>56.62</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -5929,16 +5923,16 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>HIVE</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>56.62</v>
+        <v>56.61</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -5960,16 +5954,16 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>TKR</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>56.56</v>
+        <v>56.55</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
@@ -5991,16 +5985,16 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>TKR</t>
+          <t>TNC</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>11 Robotics &amp; Physical AI / Humanoid &amp; service robot makers</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>56.55</v>
+        <v>56.09</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
@@ -6022,16 +6016,16 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>VPG</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>56.55</v>
+        <v>56.04</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
@@ -6053,16 +6047,16 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>TNC</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Humanoid &amp; service robot makers</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>56.09</v>
+        <v>56</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
@@ -6084,16 +6078,16 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>VPG</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>56.04</v>
+        <v>55.86</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
@@ -6115,16 +6109,16 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>56</v>
+        <v>55.8</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
@@ -6155,7 +6149,7 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>55.83</v>
+        <v>55.65</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
@@ -6211,7 +6205,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>55.51</v>
+        <v>55.47</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
@@ -6233,16 +6227,16 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>55.44</v>
+        <v>55.29</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
@@ -6295,21 +6289,24 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>6324.T</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>55.1</v>
+        <v>55.26</v>
       </c>
       <c r="D166" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E166" t="n">
+        <v>146</v>
       </c>
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
@@ -6319,6 +6316,34 @@
       </c>
       <c r="H166" t="inlineStr"/>
       <c r="J166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>6324.T</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr"/>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr"/>
+      <c r="J167" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
weekly-scan 2026-10-31: 48 earnings refreshes, RDDT+LRCX exit (ticket HELD), EQT-RRC merger (#240)
* weekly-scan 2026-10-31: 48 earnings refreshes, RDDT+LRCX exit (ticket HELD), EQT-RRC merger

* weekly-scan 2026-10-31: add Notion link
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-30 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-10-31 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J166"/>
+  <dimension ref="A1:J167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1068,7 +1068,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-10-30, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-10-31, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>88.7</v>
+        <v>88.62</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -1207,16 +1207,16 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>83.64</v>
+        <v>83.79000000000001</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1238,23 +1238,27 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>5.26</v>
-      </c>
-      <c r="J5" t="inlineStr"/>
+        <v>5.88</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>82.95999999999999</v>
+        <v>83.34</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1276,23 +1280,23 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>82.34999999999999</v>
+        <v>82.95999999999999</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1314,13 +1318,9 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>5.26</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
-        </is>
-      </c>
+        <v>5.88</v>
+      </c>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -1367,16 +1367,16 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>80.79000000000001</v>
+        <v>80.43000000000001</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1398,23 +1398,23 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>80.43000000000001</v>
+        <v>80.29000000000001</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1436,23 +1436,23 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>79.12</v>
+        <v>78.58</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1474,23 +1474,23 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>78.73</v>
+        <v>76.02</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1512,23 +1512,27 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.26</v>
-      </c>
-      <c r="J12" t="inlineStr"/>
+        <v>5.88</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RDDT</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>77.09999999999999</v>
+        <v>75.79000000000001</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1550,23 +1554,23 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>76.02</v>
+        <v>74.94</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1588,27 +1592,23 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.26</v>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+        <v>5.88</v>
+      </c>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>75.79000000000001</v>
+        <v>74.63</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1630,23 +1630,23 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>74.84999999999999</v>
+        <v>74.62</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1668,23 +1668,23 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 DC Infrastructure</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>74.73999999999999</v>
+        <v>74.5</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ENTER (rank 15, score 74.7)</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1706,23 +1706,23 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>03 DC Infrastructure</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>74.5</v>
+        <v>74.20999999999999</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1732,20 +1732,13 @@
       <c r="E18" t="n">
         <v>16</v>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="n">
-        <v>5.26</v>
-      </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1810,16 +1803,16 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GMED</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>73.42</v>
+        <v>73.54000000000001</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1841,23 +1834,23 @@
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="n">
-        <v>5.26</v>
+        <v>5.88</v>
       </c>
       <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>GMED</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>73.34999999999999</v>
+        <v>73.42</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1867,28 +1860,35 @@
       <c r="E22" t="n">
         <v>19</v>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>EXIT PENDING (rank 19 &gt; exit rank 18, since 2026-10-31)</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
+      <c r="I22" t="n">
+        <v>5.88</v>
+      </c>
       <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>73.16</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1910,16 +1910,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>RDDT</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>72.89</v>
+        <v>73.3</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1931,18 +1931,15 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>EXIT PENDING (rank 21 &gt; exit rank 18, since 2026-10-30)</t>
+          <t>EXIT (pending since 2026-10-30, confirmed)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="I24" t="n">
-        <v>5.26</v>
-      </c>
       <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1979,24 +1976,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>72.70999999999999</v>
+        <v>72.66</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
-      </c>
-      <c r="E26" t="n">
-        <v>23</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
@@ -2010,21 +2004,24 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>72.66</v>
+        <v>72.64</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
+      </c>
+      <c r="E27" t="n">
+        <v>23</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
@@ -2059,18 +2056,15 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>EXIT PENDING (rank 24 &gt; exit rank 18, since 2026-10-30)</t>
+          <t>EXIT (pending since 2026-10-30, confirmed)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" t="n">
-        <v>5.26</v>
-      </c>
       <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
@@ -2209,7 +2203,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>70.64</v>
+        <v>71.14</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2231,21 +2225,24 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>6954.T</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>70.63</v>
+        <v>71.09</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
+      </c>
+      <c r="E34" t="n">
+        <v>30</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
@@ -2259,24 +2256,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>6954.T</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Industrial automation &amp; robot arms</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>70.55</v>
+        <v>70.63</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
           <t>✓✓</t>
         </is>
-      </c>
-      <c r="E35" t="n">
-        <v>30</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
@@ -2318,16 +2312,16 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>70.11</v>
+        <v>70.25</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2349,20 +2343,20 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>69.91</v>
+        <v>70.11</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -2380,16 +2374,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>69.70999999999999</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2411,16 +2405,16 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>69.69</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2442,16 +2436,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>69.45</v>
+        <v>69.69</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2473,16 +2467,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>69.44</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2594,24 +2588,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>68.77</v>
+        <v>68.55</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E46" t="n">
-        <v>39</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
@@ -2625,21 +2616,24 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>68.73</v>
+        <v>68.43000000000001</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E47" t="n">
+        <v>39</v>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
@@ -2653,16 +2647,16 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>68.43000000000001</v>
+        <v>68.41</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2777,16 +2771,16 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>NOVT</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>67.73999999999999</v>
+        <v>67.69</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -2808,16 +2802,16 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>NOVT</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>67.69</v>
+        <v>67.62</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -2839,16 +2833,16 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>67.56999999999999</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2870,16 +2864,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>67.54000000000001</v>
+        <v>67.56999999999999</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2971,16 +2965,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Consumer fintech (AI adopter)</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>67.23999999999999</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -3002,16 +2996,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>67.18000000000001</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3033,16 +3027,16 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>67.15000000000001</v>
+        <v>67.14</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3064,24 +3058,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>6268.T</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>67.14</v>
+        <v>66.97</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E61" t="n">
-        <v>53</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
@@ -3095,21 +3086,24 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>6268.T</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>66.97</v>
+        <v>66.77</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E62" t="n">
+        <v>53</v>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
@@ -3123,16 +3117,16 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / Consumer fintech (AI adopter)</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>66.77</v>
+        <v>66.73999999999999</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3315,7 +3309,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>66.2</v>
+        <v>66.03</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3377,7 +3371,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>65.95</v>
+        <v>65.81</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3439,7 +3433,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>65.73</v>
+        <v>65.5</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3470,7 +3464,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>65.45</v>
+        <v>65.48999999999999</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -3492,16 +3486,16 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>65.29000000000001</v>
+        <v>65.27</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3523,16 +3517,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>65.27</v>
+        <v>65.23</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3554,16 +3548,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>GNRC</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>65.26000000000001</v>
+        <v>65.04000000000001</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3585,16 +3579,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>65.06999999999999</v>
+        <v>65.02</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3616,16 +3610,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>OUST</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>65.04000000000001</v>
+        <v>64.97</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3647,16 +3641,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>65.02</v>
+        <v>64.95</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3678,16 +3672,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>OUST</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Machine vision &amp; perception</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>64.97</v>
+        <v>64.88</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3709,16 +3703,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>64.88</v>
+        <v>64.53</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3740,21 +3734,24 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>64.5</v>
+        <v>64.48</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E83" t="n">
+        <v>73</v>
       </c>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
@@ -3785,7 +3782,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
@@ -3816,7 +3813,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
@@ -3830,16 +3827,16 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>64.33</v>
+        <v>64.27</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3847,7 +3844,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
@@ -3856,21 +3853,25 @@
         </is>
       </c>
       <c r="H86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>64.29000000000001</v>
+        <v>64.27</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3878,7 +3879,7 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
@@ -3892,16 +3893,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>PLAB</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>64.27</v>
+        <v>64.17</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3909,7 +3910,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
@@ -3918,33 +3919,26 @@
         </is>
       </c>
       <c r="H88" t="inlineStr"/>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
+      <c r="J88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>PLAB</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>64.17</v>
+        <v>64.14</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E89" t="n">
-        <v>78</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
@@ -3967,7 +3961,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>64.03</v>
+        <v>64.06</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -4099,7 +4093,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>63.48</v>
+        <v>63.51</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -4161,7 +4155,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>63.01</v>
+        <v>63.05</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -4304,12 +4298,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -4335,16 +4329,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>10 Models, Software &amp; Applications / Financial software</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>62.69</v>
+        <v>62.66</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4366,12 +4360,12 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Financial software</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -4459,16 +4453,16 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>62.44</v>
+        <v>62.33</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4490,16 +4484,16 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>62.33</v>
+        <v>62.23</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4521,16 +4515,16 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>62.25</v>
+        <v>62.06</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -4611,16 +4605,16 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>61.59</v>
+        <v>61.47</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -4642,24 +4636,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>2252.HK</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>61.48</v>
+        <v>61.14</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E112" t="n">
-        <v>99</v>
       </c>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
@@ -4673,21 +4664,24 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2252.HK</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>61.14</v>
+        <v>61.09</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E113" t="n">
+        <v>99</v>
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
@@ -4701,16 +4695,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>60.89</v>
+        <v>60.47</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4881,16 +4875,16 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>MBLY</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>60.08</v>
+        <v>59.98</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -4912,16 +4906,16 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>PRCT</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>59.99</v>
+        <v>59.95</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -4943,16 +4937,16 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>59.98</v>
+        <v>59.89</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -4974,16 +4968,16 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>PRCT</t>
+          <t>ALNT</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>59.95</v>
+        <v>59.87</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -5005,16 +4999,16 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>MBLY</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>59.87</v>
+        <v>59.86</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -5036,16 +5030,16 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>ALNT</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>59.79</v>
+        <v>59.66</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -5067,16 +5061,16 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>ASX</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>59.66</v>
+        <v>59.56</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -5098,16 +5092,16 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ASX</t>
+          <t>UCTT</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>59.56</v>
+        <v>59.17</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -5129,16 +5123,16 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>UCTT</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>59.17</v>
+        <v>59.11</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -5200,7 +5194,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>58.95</v>
+        <v>58.93</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -5346,16 +5340,16 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>58.52</v>
+        <v>58.56</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -5448,7 +5442,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>58.43</v>
+        <v>58.5</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
@@ -5470,16 +5464,16 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>AMKR</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>58.37</v>
+        <v>57.86</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
@@ -5501,16 +5495,16 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>AMKR</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>57.86</v>
+        <v>57.8</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
@@ -5532,7 +5526,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -5541,7 +5535,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>57.83</v>
+        <v>57.75</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -5563,24 +5557,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>DRO.AX</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>57.77</v>
+        <v>57.73</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E142" t="n">
-        <v>126</v>
       </c>
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
@@ -5594,7 +5585,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -5603,7 +5594,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>57.75</v>
+        <v>57.65</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -5611,7 +5602,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
@@ -5625,16 +5616,16 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>57.74</v>
+        <v>57.64</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
@@ -5642,7 +5633,7 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
@@ -5656,7 +5647,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>DRO.AX</t>
+          <t>ONDS</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -5665,12 +5656,15 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>57.73</v>
+        <v>57.53</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E145" t="n">
+        <v>128</v>
       </c>
       <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
@@ -5684,16 +5678,16 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>57.64</v>
+        <v>57.33</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
@@ -5715,16 +5709,16 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>ONDS</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>57.38</v>
+        <v>57.02</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
@@ -5746,16 +5740,16 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>PSIX</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>57.33</v>
+        <v>56.87</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
@@ -5777,16 +5771,16 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>PPL</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>57.07</v>
+        <v>56.8</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
@@ -5808,24 +5802,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>PSIX</t>
+          <t>6481.T</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>56.81</v>
+        <v>56.76</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
-      </c>
-      <c r="E150" t="n">
-        <v>133</v>
       </c>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
@@ -5839,21 +5830,24 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>6481.T</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>56.76</v>
+        <v>56.67</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E151" t="n">
+        <v>133</v>
       </c>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
@@ -5867,16 +5861,16 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>PPL</t>
+          <t>AVAV</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>56.74</v>
+        <v>56.67</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -5898,16 +5892,16 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>AVAV</t>
+          <t>HIVE</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Autonomy platforms &amp; defense</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>56.67</v>
+        <v>56.62</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -5929,16 +5923,16 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>HIVE</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>56.62</v>
+        <v>56.61</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -5960,16 +5954,16 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>TKR</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>56.56</v>
+        <v>56.55</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
@@ -5991,16 +5985,16 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>TKR</t>
+          <t>TNC</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>11 Robotics &amp; Physical AI / Humanoid &amp; service robot makers</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>56.55</v>
+        <v>56.09</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
@@ -6022,16 +6016,16 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>VPG</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>56.55</v>
+        <v>56.04</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
@@ -6053,16 +6047,16 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>TNC</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Humanoid &amp; service robot makers</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>56.09</v>
+        <v>56</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
@@ -6084,16 +6078,16 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>VPG</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>56.04</v>
+        <v>55.86</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
@@ -6115,16 +6109,16 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>56</v>
+        <v>55.8</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
@@ -6155,7 +6149,7 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>55.83</v>
+        <v>55.65</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
@@ -6211,7 +6205,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>55.51</v>
+        <v>55.47</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
@@ -6233,16 +6227,16 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>55.44</v>
+        <v>55.29</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
@@ -6295,21 +6289,24 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>6324.T</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>55.1</v>
+        <v>55.26</v>
       </c>
       <c r="D166" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
+      </c>
+      <c r="E166" t="n">
+        <v>146</v>
       </c>
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
@@ -6319,6 +6316,34 @@
       </c>
       <c r="H166" t="inlineStr"/>
       <c r="J166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>6324.T</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>11 Robotics &amp; Physical AI / Components: motion &amp; actuation</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr"/>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr"/>
+      <c r="J167" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>